<commit_message>
data: add device-state columns to scoring workbook
Adds thermal_status, battery_level_pct, and charging_state columns to Raw Scores, plus a device-state distribution diagnostic table in Summary. Recorded per MODEL_SELECTION_PROTOCOL.md 'Device state recording' -- not gated, but tracked for post-hoc correlation checks given the unresolved decoding-determinism question (ISSUE_LOG.md #12).
</commit_message>
<xml_diff>
--- a/data/model_selection/MODEL_SELECTION_SCORING.xlsx
+++ b/data/model_selection/MODEL_SELECTION_SCORING.xlsx
@@ -23,15 +23,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="97">
-  <si>
-    <t xml:space="preserve">MODEL SELECTION — MANUAL SCORING WORKBOOK</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="113">
+  <si>
+    <t xml:space="preserve">MODEL SELECTION — SCORING WORKBOOK</t>
   </si>
   <si>
     <t xml:space="preserve">Purpose</t>
   </si>
   <si>
-    <t xml:space="preserve">This workbook supports the Phase A model-feasibility evaluation (15 documents x 5 runs = 75 outputs), per MODEL_SELECTION_PROTOCOL.md. Scoring is performed manually by a bilingual (EN/FR) evaluator comparing each English source document against its French model output.</t>
+    <t xml:space="preserve">This workbook supports the Phase A model-feasibility evaluation (15 documents x 5 runs = 75 outputs), per MODEL_SELECTION_PROTOCOL.md. Scoring follows a two-step process: Claude proposes scores for each output with line-by-line justification against the source document, then the project author validates or corrects every score before it is recorded here. See MODEL_SELECTION_PROTOCOL.md, 'Scoring process' for the full rationale.</t>
   </si>
   <si>
     <t xml:space="preserve">How to use this workbook</t>
@@ -40,13 +40,19 @@
     <t xml:space="preserve">1. 'Source Documents' tab: confirm the 15 frozen documents are listed (id + file path). Optionally paste each source excerpt for quick reference while scoring.</t>
   </si>
   <si>
-    <t xml:space="preserve">2. 'Raw Scores' tab: the 75 rows (15 docs x 5 runs) are pre-generated. Paste each generated French output into the 'Output text (FR)' column, then fill in the four numeric criteria and the critical-error count.</t>
+    <t xml:space="preserve">2. 'Raw Scores' tab: the 75 rows (15 docs x 5 runs) are pre-generated. Paste each generated French output, record the device state at time of run (thermal status, battery level, charging state), then fill in the four numeric criteria and the critical-error count once validated.</t>
   </si>
   <si>
     <t xml:space="preserve">3. Only YELLOW cells should be edited. Every other cell is a formula and will recalculate automatically — do not overwrite them.</t>
   </si>
   <si>
-    <t xml:space="preserve">4. 'Summary' tab: aggregate statistics update automatically as you score. The two threshold parameters at the top (yellow) are project design decisions — set them once, before scoring begins, per §9-10 of the master prompt (do not adjust them retroactively based on results).</t>
+    <t xml:space="preserve">4. 'Summary' tab: aggregate statistics update automatically as you score. The three threshold parameters at the top (yellow) are project design decisions — set them once, before scoring begins, per §9-10 of the master prompt (do not adjust them retroactively based on results).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Device state columns</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phase A does not use the strict Phase B readiness gate (§38-43) — output content is expected to be independent of thermal/battery state under deterministic decoding. Device state is recorded (not gated) for two reasons: to allow a post-hoc check for any correlation with output anomalies, and to help identify runs that failed due to an extreme device state (excluded per §37 as an instrumentation failure, not a model-quality signal). See MODEL_SELECTION_PROTOCOL.md, 'Device state recording'.</t>
   </si>
   <si>
     <t xml:space="preserve">Scoring scale (criteria 1-4, per output)</t>
@@ -85,7 +91,7 @@
     <t xml:space="preserve">Terminology handling — are established technical terms handled appropriately (kept when conventional, explained when useful) rather than translated literally term-by-term?</t>
   </si>
   <si>
-    <t xml:space="preserve">Critical semantic errors — count of errors that invert or seriously distort meaning (e.g. negation dropped, a technical claim reversed). This is a count, not a 1-5 score.</t>
+    <t xml:space="preserve">Critical semantic errors — count of errors that invert or seriously distort meaning (e.g. negation dropped, a technical claim reversed, an unsupported relationship invented). This is a count, not a 1-5 score.</t>
   </si>
   <si>
     <t xml:space="preserve">Notes column</t>
@@ -211,6 +217,15 @@
     <t xml:space="preserve">output_text_FR</t>
   </si>
   <si>
+    <t xml:space="preserve">thermal_status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">battery_level_pct</t>
+  </si>
+  <si>
+    <t xml:space="preserve">charging_state</t>
+  </si>
+  <si>
     <t xml:space="preserve">technical_correctness (1-5)</t>
   </si>
   <si>
@@ -244,7 +259,7 @@
     <t xml:space="preserve">Per-output quality threshold (min mean_score to count as PASS)</t>
   </si>
   <si>
-    <t xml:space="preserve">Editable. Applies to each output's mean of the 4 criteria (Raw Scores col K).</t>
+    <t xml:space="preserve">Editable. Applies to each output's mean of the 4 criteria (Raw Scores col N).</t>
   </si>
   <si>
     <t xml:space="preserve">Max critical errors per output still counted as PASS</t>
@@ -314,6 +329,39 @@
   </si>
   <si>
     <t xml:space="preserve">Per-document mean (diagnostic — spot a systematically weak document)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Device state distribution (diagnostic — for post-hoc correlation checks)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thermal status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Run count</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mean score at this status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NONE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LIGHT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MODERATE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SEVERE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CRITICAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMERGENCY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SHUTDOWN</t>
   </si>
 </sst>
 </file>
@@ -783,7 +831,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A32"/>
+  <dimension ref="A1:A35"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="100"/>
@@ -802,7 +850,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
@@ -820,7 +868,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
         <v>5</v>
       </c>
@@ -843,95 +891,108 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="2"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="3" t="s">
         <v>10</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="2" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="2"/>
-    </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3" t="s">
+      <c r="A20" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="2" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="2"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="3" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="2" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="2" t="s">
         <v>18</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="2" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="2"/>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="3" t="s">
+    <row r="27" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
         <v>22</v>
       </c>
     </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="2"/>
+    </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="4" t="s">
+      <c r="A30" s="3" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="5" t="s">
+    <row r="31" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="2" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="6" t="s">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="4" t="s">
         <v>25</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="6" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -960,147 +1021,147 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C2" s="9"/>
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C3" s="9"/>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C4" s="9"/>
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C5" s="9"/>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C6" s="9"/>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C7" s="9"/>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C8" s="9"/>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C9" s="9"/>
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C10" s="9"/>
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C11" s="9"/>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C12" s="9"/>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C13" s="9"/>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="8" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C14" s="9"/>
     </row>
     <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C15" s="9"/>
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="8" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C16" s="9"/>
     </row>
@@ -1120,56 +1181,66 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L76"/>
+  <dimension ref="A1:O76"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="8"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="6" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="9" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="12"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="H1" s="7" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="I1" s="7" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="J1" s="7" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="K1" s="7" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="L1" s="7" t="s">
-        <v>69</v>
+        <v>71</v>
+      </c>
+      <c r="M1" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="N1" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="O1" s="7" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1178,7 +1249,7 @@
         <v>doc_01-R1</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C2" s="10" t="n">
         <v>1</v>
@@ -1189,13 +1260,16 @@
       <c r="G2" s="11"/>
       <c r="H2" s="11"/>
       <c r="I2" s="11"/>
-      <c r="J2" s="9"/>
-      <c r="K2" s="8" t="str">
-        <f aca="false">IF(COUNT(E2:H2)=4,AVERAGE(E2:H2),"")</f>
-        <v/>
-      </c>
-      <c r="L2" s="8" t="str">
-        <f aca="false">IF(K2="","",IF(AND(K2&gt;=Summary!$B$3,I2&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J2" s="11"/>
+      <c r="K2" s="11"/>
+      <c r="L2" s="11"/>
+      <c r="M2" s="9"/>
+      <c r="N2" s="8" t="str">
+        <f aca="false">IF(COUNT(H2:K2)=4,AVERAGE(H2:K2),"")</f>
+        <v/>
+      </c>
+      <c r="O2" s="8" t="str">
+        <f aca="false">IF(N2="","",IF(AND(N2&gt;=Summary!$B$3,L2&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -1205,7 +1279,7 @@
         <v>doc_01-R2</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C3" s="10" t="n">
         <v>2</v>
@@ -1216,13 +1290,16 @@
       <c r="G3" s="11"/>
       <c r="H3" s="11"/>
       <c r="I3" s="11"/>
-      <c r="J3" s="9"/>
-      <c r="K3" s="8" t="str">
-        <f aca="false">IF(COUNT(E3:H3)=4,AVERAGE(E3:H3),"")</f>
-        <v/>
-      </c>
-      <c r="L3" s="8" t="str">
-        <f aca="false">IF(K3="","",IF(AND(K3&gt;=Summary!$B$3,I3&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J3" s="11"/>
+      <c r="K3" s="11"/>
+      <c r="L3" s="11"/>
+      <c r="M3" s="9"/>
+      <c r="N3" s="8" t="str">
+        <f aca="false">IF(COUNT(H3:K3)=4,AVERAGE(H3:K3),"")</f>
+        <v/>
+      </c>
+      <c r="O3" s="8" t="str">
+        <f aca="false">IF(N3="","",IF(AND(N3&gt;=Summary!$B$3,L3&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -1232,7 +1309,7 @@
         <v>doc_01-R3</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C4" s="10" t="n">
         <v>3</v>
@@ -1243,13 +1320,16 @@
       <c r="G4" s="11"/>
       <c r="H4" s="11"/>
       <c r="I4" s="11"/>
-      <c r="J4" s="9"/>
-      <c r="K4" s="8" t="str">
-        <f aca="false">IF(COUNT(E4:H4)=4,AVERAGE(E4:H4),"")</f>
-        <v/>
-      </c>
-      <c r="L4" s="8" t="str">
-        <f aca="false">IF(K4="","",IF(AND(K4&gt;=Summary!$B$3,I4&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J4" s="11"/>
+      <c r="K4" s="11"/>
+      <c r="L4" s="11"/>
+      <c r="M4" s="9"/>
+      <c r="N4" s="8" t="str">
+        <f aca="false">IF(COUNT(H4:K4)=4,AVERAGE(H4:K4),"")</f>
+        <v/>
+      </c>
+      <c r="O4" s="8" t="str">
+        <f aca="false">IF(N4="","",IF(AND(N4&gt;=Summary!$B$3,L4&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -1259,7 +1339,7 @@
         <v>doc_01-R4</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C5" s="10" t="n">
         <v>4</v>
@@ -1270,13 +1350,16 @@
       <c r="G5" s="11"/>
       <c r="H5" s="11"/>
       <c r="I5" s="11"/>
-      <c r="J5" s="9"/>
-      <c r="K5" s="8" t="str">
-        <f aca="false">IF(COUNT(E5:H5)=4,AVERAGE(E5:H5),"")</f>
-        <v/>
-      </c>
-      <c r="L5" s="8" t="str">
-        <f aca="false">IF(K5="","",IF(AND(K5&gt;=Summary!$B$3,I5&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J5" s="11"/>
+      <c r="K5" s="11"/>
+      <c r="L5" s="11"/>
+      <c r="M5" s="9"/>
+      <c r="N5" s="8" t="str">
+        <f aca="false">IF(COUNT(H5:K5)=4,AVERAGE(H5:K5),"")</f>
+        <v/>
+      </c>
+      <c r="O5" s="8" t="str">
+        <f aca="false">IF(N5="","",IF(AND(N5&gt;=Summary!$B$3,L5&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -1286,7 +1369,7 @@
         <v>doc_01-R5</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C6" s="10" t="n">
         <v>5</v>
@@ -1297,13 +1380,16 @@
       <c r="G6" s="11"/>
       <c r="H6" s="11"/>
       <c r="I6" s="11"/>
-      <c r="J6" s="9"/>
-      <c r="K6" s="8" t="str">
-        <f aca="false">IF(COUNT(E6:H6)=4,AVERAGE(E6:H6),"")</f>
-        <v/>
-      </c>
-      <c r="L6" s="8" t="str">
-        <f aca="false">IF(K6="","",IF(AND(K6&gt;=Summary!$B$3,I6&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J6" s="11"/>
+      <c r="K6" s="11"/>
+      <c r="L6" s="11"/>
+      <c r="M6" s="9"/>
+      <c r="N6" s="8" t="str">
+        <f aca="false">IF(COUNT(H6:K6)=4,AVERAGE(H6:K6),"")</f>
+        <v/>
+      </c>
+      <c r="O6" s="8" t="str">
+        <f aca="false">IF(N6="","",IF(AND(N6&gt;=Summary!$B$3,L6&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -1313,7 +1399,7 @@
         <v>doc_02-R1</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C7" s="10" t="n">
         <v>1</v>
@@ -1324,13 +1410,16 @@
       <c r="G7" s="11"/>
       <c r="H7" s="11"/>
       <c r="I7" s="11"/>
-      <c r="J7" s="9"/>
-      <c r="K7" s="8" t="str">
-        <f aca="false">IF(COUNT(E7:H7)=4,AVERAGE(E7:H7),"")</f>
-        <v/>
-      </c>
-      <c r="L7" s="8" t="str">
-        <f aca="false">IF(K7="","",IF(AND(K7&gt;=Summary!$B$3,I7&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J7" s="11"/>
+      <c r="K7" s="11"/>
+      <c r="L7" s="11"/>
+      <c r="M7" s="9"/>
+      <c r="N7" s="8" t="str">
+        <f aca="false">IF(COUNT(H7:K7)=4,AVERAGE(H7:K7),"")</f>
+        <v/>
+      </c>
+      <c r="O7" s="8" t="str">
+        <f aca="false">IF(N7="","",IF(AND(N7&gt;=Summary!$B$3,L7&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -1340,7 +1429,7 @@
         <v>doc_02-R2</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C8" s="10" t="n">
         <v>2</v>
@@ -1351,13 +1440,16 @@
       <c r="G8" s="11"/>
       <c r="H8" s="11"/>
       <c r="I8" s="11"/>
-      <c r="J8" s="9"/>
-      <c r="K8" s="8" t="str">
-        <f aca="false">IF(COUNT(E8:H8)=4,AVERAGE(E8:H8),"")</f>
-        <v/>
-      </c>
-      <c r="L8" s="8" t="str">
-        <f aca="false">IF(K8="","",IF(AND(K8&gt;=Summary!$B$3,I8&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J8" s="11"/>
+      <c r="K8" s="11"/>
+      <c r="L8" s="11"/>
+      <c r="M8" s="9"/>
+      <c r="N8" s="8" t="str">
+        <f aca="false">IF(COUNT(H8:K8)=4,AVERAGE(H8:K8),"")</f>
+        <v/>
+      </c>
+      <c r="O8" s="8" t="str">
+        <f aca="false">IF(N8="","",IF(AND(N8&gt;=Summary!$B$3,L8&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -1367,7 +1459,7 @@
         <v>doc_02-R3</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C9" s="10" t="n">
         <v>3</v>
@@ -1378,13 +1470,16 @@
       <c r="G9" s="11"/>
       <c r="H9" s="11"/>
       <c r="I9" s="11"/>
-      <c r="J9" s="9"/>
-      <c r="K9" s="8" t="str">
-        <f aca="false">IF(COUNT(E9:H9)=4,AVERAGE(E9:H9),"")</f>
-        <v/>
-      </c>
-      <c r="L9" s="8" t="str">
-        <f aca="false">IF(K9="","",IF(AND(K9&gt;=Summary!$B$3,I9&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J9" s="11"/>
+      <c r="K9" s="11"/>
+      <c r="L9" s="11"/>
+      <c r="M9" s="9"/>
+      <c r="N9" s="8" t="str">
+        <f aca="false">IF(COUNT(H9:K9)=4,AVERAGE(H9:K9),"")</f>
+        <v/>
+      </c>
+      <c r="O9" s="8" t="str">
+        <f aca="false">IF(N9="","",IF(AND(N9&gt;=Summary!$B$3,L9&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -1394,7 +1489,7 @@
         <v>doc_02-R4</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C10" s="10" t="n">
         <v>4</v>
@@ -1405,13 +1500,16 @@
       <c r="G10" s="11"/>
       <c r="H10" s="11"/>
       <c r="I10" s="11"/>
-      <c r="J10" s="9"/>
-      <c r="K10" s="8" t="str">
-        <f aca="false">IF(COUNT(E10:H10)=4,AVERAGE(E10:H10),"")</f>
-        <v/>
-      </c>
-      <c r="L10" s="8" t="str">
-        <f aca="false">IF(K10="","",IF(AND(K10&gt;=Summary!$B$3,I10&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J10" s="11"/>
+      <c r="K10" s="11"/>
+      <c r="L10" s="11"/>
+      <c r="M10" s="9"/>
+      <c r="N10" s="8" t="str">
+        <f aca="false">IF(COUNT(H10:K10)=4,AVERAGE(H10:K10),"")</f>
+        <v/>
+      </c>
+      <c r="O10" s="8" t="str">
+        <f aca="false">IF(N10="","",IF(AND(N10&gt;=Summary!$B$3,L10&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -1421,7 +1519,7 @@
         <v>doc_02-R5</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C11" s="10" t="n">
         <v>5</v>
@@ -1432,13 +1530,16 @@
       <c r="G11" s="11"/>
       <c r="H11" s="11"/>
       <c r="I11" s="11"/>
-      <c r="J11" s="9"/>
-      <c r="K11" s="8" t="str">
-        <f aca="false">IF(COUNT(E11:H11)=4,AVERAGE(E11:H11),"")</f>
-        <v/>
-      </c>
-      <c r="L11" s="8" t="str">
-        <f aca="false">IF(K11="","",IF(AND(K11&gt;=Summary!$B$3,I11&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J11" s="11"/>
+      <c r="K11" s="11"/>
+      <c r="L11" s="11"/>
+      <c r="M11" s="9"/>
+      <c r="N11" s="8" t="str">
+        <f aca="false">IF(COUNT(H11:K11)=4,AVERAGE(H11:K11),"")</f>
+        <v/>
+      </c>
+      <c r="O11" s="8" t="str">
+        <f aca="false">IF(N11="","",IF(AND(N11&gt;=Summary!$B$3,L11&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -1448,7 +1549,7 @@
         <v>doc_03-R1</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C12" s="10" t="n">
         <v>1</v>
@@ -1459,13 +1560,16 @@
       <c r="G12" s="11"/>
       <c r="H12" s="11"/>
       <c r="I12" s="11"/>
-      <c r="J12" s="9"/>
-      <c r="K12" s="8" t="str">
-        <f aca="false">IF(COUNT(E12:H12)=4,AVERAGE(E12:H12),"")</f>
-        <v/>
-      </c>
-      <c r="L12" s="8" t="str">
-        <f aca="false">IF(K12="","",IF(AND(K12&gt;=Summary!$B$3,I12&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J12" s="11"/>
+      <c r="K12" s="11"/>
+      <c r="L12" s="11"/>
+      <c r="M12" s="9"/>
+      <c r="N12" s="8" t="str">
+        <f aca="false">IF(COUNT(H12:K12)=4,AVERAGE(H12:K12),"")</f>
+        <v/>
+      </c>
+      <c r="O12" s="8" t="str">
+        <f aca="false">IF(N12="","",IF(AND(N12&gt;=Summary!$B$3,L12&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -1475,7 +1579,7 @@
         <v>doc_03-R2</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C13" s="10" t="n">
         <v>2</v>
@@ -1486,13 +1590,16 @@
       <c r="G13" s="11"/>
       <c r="H13" s="11"/>
       <c r="I13" s="11"/>
-      <c r="J13" s="9"/>
-      <c r="K13" s="8" t="str">
-        <f aca="false">IF(COUNT(E13:H13)=4,AVERAGE(E13:H13),"")</f>
-        <v/>
-      </c>
-      <c r="L13" s="8" t="str">
-        <f aca="false">IF(K13="","",IF(AND(K13&gt;=Summary!$B$3,I13&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J13" s="11"/>
+      <c r="K13" s="11"/>
+      <c r="L13" s="11"/>
+      <c r="M13" s="9"/>
+      <c r="N13" s="8" t="str">
+        <f aca="false">IF(COUNT(H13:K13)=4,AVERAGE(H13:K13),"")</f>
+        <v/>
+      </c>
+      <c r="O13" s="8" t="str">
+        <f aca="false">IF(N13="","",IF(AND(N13&gt;=Summary!$B$3,L13&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -1502,7 +1609,7 @@
         <v>doc_03-R3</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C14" s="10" t="n">
         <v>3</v>
@@ -1513,13 +1620,16 @@
       <c r="G14" s="11"/>
       <c r="H14" s="11"/>
       <c r="I14" s="11"/>
-      <c r="J14" s="9"/>
-      <c r="K14" s="8" t="str">
-        <f aca="false">IF(COUNT(E14:H14)=4,AVERAGE(E14:H14),"")</f>
-        <v/>
-      </c>
-      <c r="L14" s="8" t="str">
-        <f aca="false">IF(K14="","",IF(AND(K14&gt;=Summary!$B$3,I14&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J14" s="11"/>
+      <c r="K14" s="11"/>
+      <c r="L14" s="11"/>
+      <c r="M14" s="9"/>
+      <c r="N14" s="8" t="str">
+        <f aca="false">IF(COUNT(H14:K14)=4,AVERAGE(H14:K14),"")</f>
+        <v/>
+      </c>
+      <c r="O14" s="8" t="str">
+        <f aca="false">IF(N14="","",IF(AND(N14&gt;=Summary!$B$3,L14&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -1529,7 +1639,7 @@
         <v>doc_03-R4</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C15" s="10" t="n">
         <v>4</v>
@@ -1540,13 +1650,16 @@
       <c r="G15" s="11"/>
       <c r="H15" s="11"/>
       <c r="I15" s="11"/>
-      <c r="J15" s="9"/>
-      <c r="K15" s="8" t="str">
-        <f aca="false">IF(COUNT(E15:H15)=4,AVERAGE(E15:H15),"")</f>
-        <v/>
-      </c>
-      <c r="L15" s="8" t="str">
-        <f aca="false">IF(K15="","",IF(AND(K15&gt;=Summary!$B$3,I15&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J15" s="11"/>
+      <c r="K15" s="11"/>
+      <c r="L15" s="11"/>
+      <c r="M15" s="9"/>
+      <c r="N15" s="8" t="str">
+        <f aca="false">IF(COUNT(H15:K15)=4,AVERAGE(H15:K15),"")</f>
+        <v/>
+      </c>
+      <c r="O15" s="8" t="str">
+        <f aca="false">IF(N15="","",IF(AND(N15&gt;=Summary!$B$3,L15&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -1556,7 +1669,7 @@
         <v>doc_03-R5</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C16" s="10" t="n">
         <v>5</v>
@@ -1567,13 +1680,16 @@
       <c r="G16" s="11"/>
       <c r="H16" s="11"/>
       <c r="I16" s="11"/>
-      <c r="J16" s="9"/>
-      <c r="K16" s="8" t="str">
-        <f aca="false">IF(COUNT(E16:H16)=4,AVERAGE(E16:H16),"")</f>
-        <v/>
-      </c>
-      <c r="L16" s="8" t="str">
-        <f aca="false">IF(K16="","",IF(AND(K16&gt;=Summary!$B$3,I16&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J16" s="11"/>
+      <c r="K16" s="11"/>
+      <c r="L16" s="11"/>
+      <c r="M16" s="9"/>
+      <c r="N16" s="8" t="str">
+        <f aca="false">IF(COUNT(H16:K16)=4,AVERAGE(H16:K16),"")</f>
+        <v/>
+      </c>
+      <c r="O16" s="8" t="str">
+        <f aca="false">IF(N16="","",IF(AND(N16&gt;=Summary!$B$3,L16&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -1583,7 +1699,7 @@
         <v>doc_04-R1</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C17" s="10" t="n">
         <v>1</v>
@@ -1594,13 +1710,16 @@
       <c r="G17" s="11"/>
       <c r="H17" s="11"/>
       <c r="I17" s="11"/>
-      <c r="J17" s="9"/>
-      <c r="K17" s="8" t="str">
-        <f aca="false">IF(COUNT(E17:H17)=4,AVERAGE(E17:H17),"")</f>
-        <v/>
-      </c>
-      <c r="L17" s="8" t="str">
-        <f aca="false">IF(K17="","",IF(AND(K17&gt;=Summary!$B$3,I17&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J17" s="11"/>
+      <c r="K17" s="11"/>
+      <c r="L17" s="11"/>
+      <c r="M17" s="9"/>
+      <c r="N17" s="8" t="str">
+        <f aca="false">IF(COUNT(H17:K17)=4,AVERAGE(H17:K17),"")</f>
+        <v/>
+      </c>
+      <c r="O17" s="8" t="str">
+        <f aca="false">IF(N17="","",IF(AND(N17&gt;=Summary!$B$3,L17&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -1610,7 +1729,7 @@
         <v>doc_04-R2</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C18" s="10" t="n">
         <v>2</v>
@@ -1621,13 +1740,16 @@
       <c r="G18" s="11"/>
       <c r="H18" s="11"/>
       <c r="I18" s="11"/>
-      <c r="J18" s="9"/>
-      <c r="K18" s="8" t="str">
-        <f aca="false">IF(COUNT(E18:H18)=4,AVERAGE(E18:H18),"")</f>
-        <v/>
-      </c>
-      <c r="L18" s="8" t="str">
-        <f aca="false">IF(K18="","",IF(AND(K18&gt;=Summary!$B$3,I18&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J18" s="11"/>
+      <c r="K18" s="11"/>
+      <c r="L18" s="11"/>
+      <c r="M18" s="9"/>
+      <c r="N18" s="8" t="str">
+        <f aca="false">IF(COUNT(H18:K18)=4,AVERAGE(H18:K18),"")</f>
+        <v/>
+      </c>
+      <c r="O18" s="8" t="str">
+        <f aca="false">IF(N18="","",IF(AND(N18&gt;=Summary!$B$3,L18&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -1637,7 +1759,7 @@
         <v>doc_04-R3</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C19" s="10" t="n">
         <v>3</v>
@@ -1648,13 +1770,16 @@
       <c r="G19" s="11"/>
       <c r="H19" s="11"/>
       <c r="I19" s="11"/>
-      <c r="J19" s="9"/>
-      <c r="K19" s="8" t="str">
-        <f aca="false">IF(COUNT(E19:H19)=4,AVERAGE(E19:H19),"")</f>
-        <v/>
-      </c>
-      <c r="L19" s="8" t="str">
-        <f aca="false">IF(K19="","",IF(AND(K19&gt;=Summary!$B$3,I19&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J19" s="11"/>
+      <c r="K19" s="11"/>
+      <c r="L19" s="11"/>
+      <c r="M19" s="9"/>
+      <c r="N19" s="8" t="str">
+        <f aca="false">IF(COUNT(H19:K19)=4,AVERAGE(H19:K19),"")</f>
+        <v/>
+      </c>
+      <c r="O19" s="8" t="str">
+        <f aca="false">IF(N19="","",IF(AND(N19&gt;=Summary!$B$3,L19&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -1664,7 +1789,7 @@
         <v>doc_04-R4</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C20" s="10" t="n">
         <v>4</v>
@@ -1675,13 +1800,16 @@
       <c r="G20" s="11"/>
       <c r="H20" s="11"/>
       <c r="I20" s="11"/>
-      <c r="J20" s="9"/>
-      <c r="K20" s="8" t="str">
-        <f aca="false">IF(COUNT(E20:H20)=4,AVERAGE(E20:H20),"")</f>
-        <v/>
-      </c>
-      <c r="L20" s="8" t="str">
-        <f aca="false">IF(K20="","",IF(AND(K20&gt;=Summary!$B$3,I20&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J20" s="11"/>
+      <c r="K20" s="11"/>
+      <c r="L20" s="11"/>
+      <c r="M20" s="9"/>
+      <c r="N20" s="8" t="str">
+        <f aca="false">IF(COUNT(H20:K20)=4,AVERAGE(H20:K20),"")</f>
+        <v/>
+      </c>
+      <c r="O20" s="8" t="str">
+        <f aca="false">IF(N20="","",IF(AND(N20&gt;=Summary!$B$3,L20&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -1691,7 +1819,7 @@
         <v>doc_04-R5</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C21" s="10" t="n">
         <v>5</v>
@@ -1702,13 +1830,16 @@
       <c r="G21" s="11"/>
       <c r="H21" s="11"/>
       <c r="I21" s="11"/>
-      <c r="J21" s="9"/>
-      <c r="K21" s="8" t="str">
-        <f aca="false">IF(COUNT(E21:H21)=4,AVERAGE(E21:H21),"")</f>
-        <v/>
-      </c>
-      <c r="L21" s="8" t="str">
-        <f aca="false">IF(K21="","",IF(AND(K21&gt;=Summary!$B$3,I21&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J21" s="11"/>
+      <c r="K21" s="11"/>
+      <c r="L21" s="11"/>
+      <c r="M21" s="9"/>
+      <c r="N21" s="8" t="str">
+        <f aca="false">IF(COUNT(H21:K21)=4,AVERAGE(H21:K21),"")</f>
+        <v/>
+      </c>
+      <c r="O21" s="8" t="str">
+        <f aca="false">IF(N21="","",IF(AND(N21&gt;=Summary!$B$3,L21&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -1718,7 +1849,7 @@
         <v>doc_05-R1</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C22" s="10" t="n">
         <v>1</v>
@@ -1729,13 +1860,16 @@
       <c r="G22" s="11"/>
       <c r="H22" s="11"/>
       <c r="I22" s="11"/>
-      <c r="J22" s="9"/>
-      <c r="K22" s="8" t="str">
-        <f aca="false">IF(COUNT(E22:H22)=4,AVERAGE(E22:H22),"")</f>
-        <v/>
-      </c>
-      <c r="L22" s="8" t="str">
-        <f aca="false">IF(K22="","",IF(AND(K22&gt;=Summary!$B$3,I22&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J22" s="11"/>
+      <c r="K22" s="11"/>
+      <c r="L22" s="11"/>
+      <c r="M22" s="9"/>
+      <c r="N22" s="8" t="str">
+        <f aca="false">IF(COUNT(H22:K22)=4,AVERAGE(H22:K22),"")</f>
+        <v/>
+      </c>
+      <c r="O22" s="8" t="str">
+        <f aca="false">IF(N22="","",IF(AND(N22&gt;=Summary!$B$3,L22&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -1745,7 +1879,7 @@
         <v>doc_05-R2</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C23" s="10" t="n">
         <v>2</v>
@@ -1756,13 +1890,16 @@
       <c r="G23" s="11"/>
       <c r="H23" s="11"/>
       <c r="I23" s="11"/>
-      <c r="J23" s="9"/>
-      <c r="K23" s="8" t="str">
-        <f aca="false">IF(COUNT(E23:H23)=4,AVERAGE(E23:H23),"")</f>
-        <v/>
-      </c>
-      <c r="L23" s="8" t="str">
-        <f aca="false">IF(K23="","",IF(AND(K23&gt;=Summary!$B$3,I23&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J23" s="11"/>
+      <c r="K23" s="11"/>
+      <c r="L23" s="11"/>
+      <c r="M23" s="9"/>
+      <c r="N23" s="8" t="str">
+        <f aca="false">IF(COUNT(H23:K23)=4,AVERAGE(H23:K23),"")</f>
+        <v/>
+      </c>
+      <c r="O23" s="8" t="str">
+        <f aca="false">IF(N23="","",IF(AND(N23&gt;=Summary!$B$3,L23&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -1772,7 +1909,7 @@
         <v>doc_05-R3</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C24" s="10" t="n">
         <v>3</v>
@@ -1783,13 +1920,16 @@
       <c r="G24" s="11"/>
       <c r="H24" s="11"/>
       <c r="I24" s="11"/>
-      <c r="J24" s="9"/>
-      <c r="K24" s="8" t="str">
-        <f aca="false">IF(COUNT(E24:H24)=4,AVERAGE(E24:H24),"")</f>
-        <v/>
-      </c>
-      <c r="L24" s="8" t="str">
-        <f aca="false">IF(K24="","",IF(AND(K24&gt;=Summary!$B$3,I24&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J24" s="11"/>
+      <c r="K24" s="11"/>
+      <c r="L24" s="11"/>
+      <c r="M24" s="9"/>
+      <c r="N24" s="8" t="str">
+        <f aca="false">IF(COUNT(H24:K24)=4,AVERAGE(H24:K24),"")</f>
+        <v/>
+      </c>
+      <c r="O24" s="8" t="str">
+        <f aca="false">IF(N24="","",IF(AND(N24&gt;=Summary!$B$3,L24&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -1799,7 +1939,7 @@
         <v>doc_05-R4</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C25" s="10" t="n">
         <v>4</v>
@@ -1810,13 +1950,16 @@
       <c r="G25" s="11"/>
       <c r="H25" s="11"/>
       <c r="I25" s="11"/>
-      <c r="J25" s="9"/>
-      <c r="K25" s="8" t="str">
-        <f aca="false">IF(COUNT(E25:H25)=4,AVERAGE(E25:H25),"")</f>
-        <v/>
-      </c>
-      <c r="L25" s="8" t="str">
-        <f aca="false">IF(K25="","",IF(AND(K25&gt;=Summary!$B$3,I25&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J25" s="11"/>
+      <c r="K25" s="11"/>
+      <c r="L25" s="11"/>
+      <c r="M25" s="9"/>
+      <c r="N25" s="8" t="str">
+        <f aca="false">IF(COUNT(H25:K25)=4,AVERAGE(H25:K25),"")</f>
+        <v/>
+      </c>
+      <c r="O25" s="8" t="str">
+        <f aca="false">IF(N25="","",IF(AND(N25&gt;=Summary!$B$3,L25&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -1826,7 +1969,7 @@
         <v>doc_05-R5</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C26" s="10" t="n">
         <v>5</v>
@@ -1837,13 +1980,16 @@
       <c r="G26" s="11"/>
       <c r="H26" s="11"/>
       <c r="I26" s="11"/>
-      <c r="J26" s="9"/>
-      <c r="K26" s="8" t="str">
-        <f aca="false">IF(COUNT(E26:H26)=4,AVERAGE(E26:H26),"")</f>
-        <v/>
-      </c>
-      <c r="L26" s="8" t="str">
-        <f aca="false">IF(K26="","",IF(AND(K26&gt;=Summary!$B$3,I26&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J26" s="11"/>
+      <c r="K26" s="11"/>
+      <c r="L26" s="11"/>
+      <c r="M26" s="9"/>
+      <c r="N26" s="8" t="str">
+        <f aca="false">IF(COUNT(H26:K26)=4,AVERAGE(H26:K26),"")</f>
+        <v/>
+      </c>
+      <c r="O26" s="8" t="str">
+        <f aca="false">IF(N26="","",IF(AND(N26&gt;=Summary!$B$3,L26&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -1853,7 +1999,7 @@
         <v>doc_06-R1</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C27" s="10" t="n">
         <v>1</v>
@@ -1864,13 +2010,16 @@
       <c r="G27" s="11"/>
       <c r="H27" s="11"/>
       <c r="I27" s="11"/>
-      <c r="J27" s="9"/>
-      <c r="K27" s="8" t="str">
-        <f aca="false">IF(COUNT(E27:H27)=4,AVERAGE(E27:H27),"")</f>
-        <v/>
-      </c>
-      <c r="L27" s="8" t="str">
-        <f aca="false">IF(K27="","",IF(AND(K27&gt;=Summary!$B$3,I27&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J27" s="11"/>
+      <c r="K27" s="11"/>
+      <c r="L27" s="11"/>
+      <c r="M27" s="9"/>
+      <c r="N27" s="8" t="str">
+        <f aca="false">IF(COUNT(H27:K27)=4,AVERAGE(H27:K27),"")</f>
+        <v/>
+      </c>
+      <c r="O27" s="8" t="str">
+        <f aca="false">IF(N27="","",IF(AND(N27&gt;=Summary!$B$3,L27&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -1880,7 +2029,7 @@
         <v>doc_06-R2</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C28" s="10" t="n">
         <v>2</v>
@@ -1891,13 +2040,16 @@
       <c r="G28" s="11"/>
       <c r="H28" s="11"/>
       <c r="I28" s="11"/>
-      <c r="J28" s="9"/>
-      <c r="K28" s="8" t="str">
-        <f aca="false">IF(COUNT(E28:H28)=4,AVERAGE(E28:H28),"")</f>
-        <v/>
-      </c>
-      <c r="L28" s="8" t="str">
-        <f aca="false">IF(K28="","",IF(AND(K28&gt;=Summary!$B$3,I28&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J28" s="11"/>
+      <c r="K28" s="11"/>
+      <c r="L28" s="11"/>
+      <c r="M28" s="9"/>
+      <c r="N28" s="8" t="str">
+        <f aca="false">IF(COUNT(H28:K28)=4,AVERAGE(H28:K28),"")</f>
+        <v/>
+      </c>
+      <c r="O28" s="8" t="str">
+        <f aca="false">IF(N28="","",IF(AND(N28&gt;=Summary!$B$3,L28&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -1907,7 +2059,7 @@
         <v>doc_06-R3</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C29" s="10" t="n">
         <v>3</v>
@@ -1918,13 +2070,16 @@
       <c r="G29" s="11"/>
       <c r="H29" s="11"/>
       <c r="I29" s="11"/>
-      <c r="J29" s="9"/>
-      <c r="K29" s="8" t="str">
-        <f aca="false">IF(COUNT(E29:H29)=4,AVERAGE(E29:H29),"")</f>
-        <v/>
-      </c>
-      <c r="L29" s="8" t="str">
-        <f aca="false">IF(K29="","",IF(AND(K29&gt;=Summary!$B$3,I29&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J29" s="11"/>
+      <c r="K29" s="11"/>
+      <c r="L29" s="11"/>
+      <c r="M29" s="9"/>
+      <c r="N29" s="8" t="str">
+        <f aca="false">IF(COUNT(H29:K29)=4,AVERAGE(H29:K29),"")</f>
+        <v/>
+      </c>
+      <c r="O29" s="8" t="str">
+        <f aca="false">IF(N29="","",IF(AND(N29&gt;=Summary!$B$3,L29&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -1934,7 +2089,7 @@
         <v>doc_06-R4</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C30" s="10" t="n">
         <v>4</v>
@@ -1945,13 +2100,16 @@
       <c r="G30" s="11"/>
       <c r="H30" s="11"/>
       <c r="I30" s="11"/>
-      <c r="J30" s="9"/>
-      <c r="K30" s="8" t="str">
-        <f aca="false">IF(COUNT(E30:H30)=4,AVERAGE(E30:H30),"")</f>
-        <v/>
-      </c>
-      <c r="L30" s="8" t="str">
-        <f aca="false">IF(K30="","",IF(AND(K30&gt;=Summary!$B$3,I30&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J30" s="11"/>
+      <c r="K30" s="11"/>
+      <c r="L30" s="11"/>
+      <c r="M30" s="9"/>
+      <c r="N30" s="8" t="str">
+        <f aca="false">IF(COUNT(H30:K30)=4,AVERAGE(H30:K30),"")</f>
+        <v/>
+      </c>
+      <c r="O30" s="8" t="str">
+        <f aca="false">IF(N30="","",IF(AND(N30&gt;=Summary!$B$3,L30&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -1961,7 +2119,7 @@
         <v>doc_06-R5</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C31" s="10" t="n">
         <v>5</v>
@@ -1972,13 +2130,16 @@
       <c r="G31" s="11"/>
       <c r="H31" s="11"/>
       <c r="I31" s="11"/>
-      <c r="J31" s="9"/>
-      <c r="K31" s="8" t="str">
-        <f aca="false">IF(COUNT(E31:H31)=4,AVERAGE(E31:H31),"")</f>
-        <v/>
-      </c>
-      <c r="L31" s="8" t="str">
-        <f aca="false">IF(K31="","",IF(AND(K31&gt;=Summary!$B$3,I31&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J31" s="11"/>
+      <c r="K31" s="11"/>
+      <c r="L31" s="11"/>
+      <c r="M31" s="9"/>
+      <c r="N31" s="8" t="str">
+        <f aca="false">IF(COUNT(H31:K31)=4,AVERAGE(H31:K31),"")</f>
+        <v/>
+      </c>
+      <c r="O31" s="8" t="str">
+        <f aca="false">IF(N31="","",IF(AND(N31&gt;=Summary!$B$3,L31&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -1988,7 +2149,7 @@
         <v>doc_07-R1</v>
       </c>
       <c r="B32" s="10" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C32" s="10" t="n">
         <v>1</v>
@@ -1999,13 +2160,16 @@
       <c r="G32" s="11"/>
       <c r="H32" s="11"/>
       <c r="I32" s="11"/>
-      <c r="J32" s="9"/>
-      <c r="K32" s="8" t="str">
-        <f aca="false">IF(COUNT(E32:H32)=4,AVERAGE(E32:H32),"")</f>
-        <v/>
-      </c>
-      <c r="L32" s="8" t="str">
-        <f aca="false">IF(K32="","",IF(AND(K32&gt;=Summary!$B$3,I32&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J32" s="11"/>
+      <c r="K32" s="11"/>
+      <c r="L32" s="11"/>
+      <c r="M32" s="9"/>
+      <c r="N32" s="8" t="str">
+        <f aca="false">IF(COUNT(H32:K32)=4,AVERAGE(H32:K32),"")</f>
+        <v/>
+      </c>
+      <c r="O32" s="8" t="str">
+        <f aca="false">IF(N32="","",IF(AND(N32&gt;=Summary!$B$3,L32&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -2015,7 +2179,7 @@
         <v>doc_07-R2</v>
       </c>
       <c r="B33" s="10" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C33" s="10" t="n">
         <v>2</v>
@@ -2026,13 +2190,16 @@
       <c r="G33" s="11"/>
       <c r="H33" s="11"/>
       <c r="I33" s="11"/>
-      <c r="J33" s="9"/>
-      <c r="K33" s="8" t="str">
-        <f aca="false">IF(COUNT(E33:H33)=4,AVERAGE(E33:H33),"")</f>
-        <v/>
-      </c>
-      <c r="L33" s="8" t="str">
-        <f aca="false">IF(K33="","",IF(AND(K33&gt;=Summary!$B$3,I33&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J33" s="11"/>
+      <c r="K33" s="11"/>
+      <c r="L33" s="11"/>
+      <c r="M33" s="9"/>
+      <c r="N33" s="8" t="str">
+        <f aca="false">IF(COUNT(H33:K33)=4,AVERAGE(H33:K33),"")</f>
+        <v/>
+      </c>
+      <c r="O33" s="8" t="str">
+        <f aca="false">IF(N33="","",IF(AND(N33&gt;=Summary!$B$3,L33&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -2042,7 +2209,7 @@
         <v>doc_07-R3</v>
       </c>
       <c r="B34" s="10" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C34" s="10" t="n">
         <v>3</v>
@@ -2053,13 +2220,16 @@
       <c r="G34" s="11"/>
       <c r="H34" s="11"/>
       <c r="I34" s="11"/>
-      <c r="J34" s="9"/>
-      <c r="K34" s="8" t="str">
-        <f aca="false">IF(COUNT(E34:H34)=4,AVERAGE(E34:H34),"")</f>
-        <v/>
-      </c>
-      <c r="L34" s="8" t="str">
-        <f aca="false">IF(K34="","",IF(AND(K34&gt;=Summary!$B$3,I34&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J34" s="11"/>
+      <c r="K34" s="11"/>
+      <c r="L34" s="11"/>
+      <c r="M34" s="9"/>
+      <c r="N34" s="8" t="str">
+        <f aca="false">IF(COUNT(H34:K34)=4,AVERAGE(H34:K34),"")</f>
+        <v/>
+      </c>
+      <c r="O34" s="8" t="str">
+        <f aca="false">IF(N34="","",IF(AND(N34&gt;=Summary!$B$3,L34&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -2069,7 +2239,7 @@
         <v>doc_07-R4</v>
       </c>
       <c r="B35" s="10" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C35" s="10" t="n">
         <v>4</v>
@@ -2080,13 +2250,16 @@
       <c r="G35" s="11"/>
       <c r="H35" s="11"/>
       <c r="I35" s="11"/>
-      <c r="J35" s="9"/>
-      <c r="K35" s="8" t="str">
-        <f aca="false">IF(COUNT(E35:H35)=4,AVERAGE(E35:H35),"")</f>
-        <v/>
-      </c>
-      <c r="L35" s="8" t="str">
-        <f aca="false">IF(K35="","",IF(AND(K35&gt;=Summary!$B$3,I35&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J35" s="11"/>
+      <c r="K35" s="11"/>
+      <c r="L35" s="11"/>
+      <c r="M35" s="9"/>
+      <c r="N35" s="8" t="str">
+        <f aca="false">IF(COUNT(H35:K35)=4,AVERAGE(H35:K35),"")</f>
+        <v/>
+      </c>
+      <c r="O35" s="8" t="str">
+        <f aca="false">IF(N35="","",IF(AND(N35&gt;=Summary!$B$3,L35&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -2096,7 +2269,7 @@
         <v>doc_07-R5</v>
       </c>
       <c r="B36" s="10" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C36" s="10" t="n">
         <v>5</v>
@@ -2107,13 +2280,16 @@
       <c r="G36" s="11"/>
       <c r="H36" s="11"/>
       <c r="I36" s="11"/>
-      <c r="J36" s="9"/>
-      <c r="K36" s="8" t="str">
-        <f aca="false">IF(COUNT(E36:H36)=4,AVERAGE(E36:H36),"")</f>
-        <v/>
-      </c>
-      <c r="L36" s="8" t="str">
-        <f aca="false">IF(K36="","",IF(AND(K36&gt;=Summary!$B$3,I36&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J36" s="11"/>
+      <c r="K36" s="11"/>
+      <c r="L36" s="11"/>
+      <c r="M36" s="9"/>
+      <c r="N36" s="8" t="str">
+        <f aca="false">IF(COUNT(H36:K36)=4,AVERAGE(H36:K36),"")</f>
+        <v/>
+      </c>
+      <c r="O36" s="8" t="str">
+        <f aca="false">IF(N36="","",IF(AND(N36&gt;=Summary!$B$3,L36&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -2123,7 +2299,7 @@
         <v>doc_08-R1</v>
       </c>
       <c r="B37" s="10" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C37" s="10" t="n">
         <v>1</v>
@@ -2134,13 +2310,16 @@
       <c r="G37" s="11"/>
       <c r="H37" s="11"/>
       <c r="I37" s="11"/>
-      <c r="J37" s="9"/>
-      <c r="K37" s="8" t="str">
-        <f aca="false">IF(COUNT(E37:H37)=4,AVERAGE(E37:H37),"")</f>
-        <v/>
-      </c>
-      <c r="L37" s="8" t="str">
-        <f aca="false">IF(K37="","",IF(AND(K37&gt;=Summary!$B$3,I37&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J37" s="11"/>
+      <c r="K37" s="11"/>
+      <c r="L37" s="11"/>
+      <c r="M37" s="9"/>
+      <c r="N37" s="8" t="str">
+        <f aca="false">IF(COUNT(H37:K37)=4,AVERAGE(H37:K37),"")</f>
+        <v/>
+      </c>
+      <c r="O37" s="8" t="str">
+        <f aca="false">IF(N37="","",IF(AND(N37&gt;=Summary!$B$3,L37&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -2150,7 +2329,7 @@
         <v>doc_08-R2</v>
       </c>
       <c r="B38" s="10" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C38" s="10" t="n">
         <v>2</v>
@@ -2161,13 +2340,16 @@
       <c r="G38" s="11"/>
       <c r="H38" s="11"/>
       <c r="I38" s="11"/>
-      <c r="J38" s="9"/>
-      <c r="K38" s="8" t="str">
-        <f aca="false">IF(COUNT(E38:H38)=4,AVERAGE(E38:H38),"")</f>
-        <v/>
-      </c>
-      <c r="L38" s="8" t="str">
-        <f aca="false">IF(K38="","",IF(AND(K38&gt;=Summary!$B$3,I38&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J38" s="11"/>
+      <c r="K38" s="11"/>
+      <c r="L38" s="11"/>
+      <c r="M38" s="9"/>
+      <c r="N38" s="8" t="str">
+        <f aca="false">IF(COUNT(H38:K38)=4,AVERAGE(H38:K38),"")</f>
+        <v/>
+      </c>
+      <c r="O38" s="8" t="str">
+        <f aca="false">IF(N38="","",IF(AND(N38&gt;=Summary!$B$3,L38&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -2177,7 +2359,7 @@
         <v>doc_08-R3</v>
       </c>
       <c r="B39" s="10" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C39" s="10" t="n">
         <v>3</v>
@@ -2188,13 +2370,16 @@
       <c r="G39" s="11"/>
       <c r="H39" s="11"/>
       <c r="I39" s="11"/>
-      <c r="J39" s="9"/>
-      <c r="K39" s="8" t="str">
-        <f aca="false">IF(COUNT(E39:H39)=4,AVERAGE(E39:H39),"")</f>
-        <v/>
-      </c>
-      <c r="L39" s="8" t="str">
-        <f aca="false">IF(K39="","",IF(AND(K39&gt;=Summary!$B$3,I39&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J39" s="11"/>
+      <c r="K39" s="11"/>
+      <c r="L39" s="11"/>
+      <c r="M39" s="9"/>
+      <c r="N39" s="8" t="str">
+        <f aca="false">IF(COUNT(H39:K39)=4,AVERAGE(H39:K39),"")</f>
+        <v/>
+      </c>
+      <c r="O39" s="8" t="str">
+        <f aca="false">IF(N39="","",IF(AND(N39&gt;=Summary!$B$3,L39&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -2204,7 +2389,7 @@
         <v>doc_08-R4</v>
       </c>
       <c r="B40" s="10" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C40" s="10" t="n">
         <v>4</v>
@@ -2215,13 +2400,16 @@
       <c r="G40" s="11"/>
       <c r="H40" s="11"/>
       <c r="I40" s="11"/>
-      <c r="J40" s="9"/>
-      <c r="K40" s="8" t="str">
-        <f aca="false">IF(COUNT(E40:H40)=4,AVERAGE(E40:H40),"")</f>
-        <v/>
-      </c>
-      <c r="L40" s="8" t="str">
-        <f aca="false">IF(K40="","",IF(AND(K40&gt;=Summary!$B$3,I40&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J40" s="11"/>
+      <c r="K40" s="11"/>
+      <c r="L40" s="11"/>
+      <c r="M40" s="9"/>
+      <c r="N40" s="8" t="str">
+        <f aca="false">IF(COUNT(H40:K40)=4,AVERAGE(H40:K40),"")</f>
+        <v/>
+      </c>
+      <c r="O40" s="8" t="str">
+        <f aca="false">IF(N40="","",IF(AND(N40&gt;=Summary!$B$3,L40&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -2231,7 +2419,7 @@
         <v>doc_08-R5</v>
       </c>
       <c r="B41" s="10" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C41" s="10" t="n">
         <v>5</v>
@@ -2242,13 +2430,16 @@
       <c r="G41" s="11"/>
       <c r="H41" s="11"/>
       <c r="I41" s="11"/>
-      <c r="J41" s="9"/>
-      <c r="K41" s="8" t="str">
-        <f aca="false">IF(COUNT(E41:H41)=4,AVERAGE(E41:H41),"")</f>
-        <v/>
-      </c>
-      <c r="L41" s="8" t="str">
-        <f aca="false">IF(K41="","",IF(AND(K41&gt;=Summary!$B$3,I41&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J41" s="11"/>
+      <c r="K41" s="11"/>
+      <c r="L41" s="11"/>
+      <c r="M41" s="9"/>
+      <c r="N41" s="8" t="str">
+        <f aca="false">IF(COUNT(H41:K41)=4,AVERAGE(H41:K41),"")</f>
+        <v/>
+      </c>
+      <c r="O41" s="8" t="str">
+        <f aca="false">IF(N41="","",IF(AND(N41&gt;=Summary!$B$3,L41&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -2258,7 +2449,7 @@
         <v>doc_09-R1</v>
       </c>
       <c r="B42" s="10" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C42" s="10" t="n">
         <v>1</v>
@@ -2269,13 +2460,16 @@
       <c r="G42" s="11"/>
       <c r="H42" s="11"/>
       <c r="I42" s="11"/>
-      <c r="J42" s="9"/>
-      <c r="K42" s="8" t="str">
-        <f aca="false">IF(COUNT(E42:H42)=4,AVERAGE(E42:H42),"")</f>
-        <v/>
-      </c>
-      <c r="L42" s="8" t="str">
-        <f aca="false">IF(K42="","",IF(AND(K42&gt;=Summary!$B$3,I42&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J42" s="11"/>
+      <c r="K42" s="11"/>
+      <c r="L42" s="11"/>
+      <c r="M42" s="9"/>
+      <c r="N42" s="8" t="str">
+        <f aca="false">IF(COUNT(H42:K42)=4,AVERAGE(H42:K42),"")</f>
+        <v/>
+      </c>
+      <c r="O42" s="8" t="str">
+        <f aca="false">IF(N42="","",IF(AND(N42&gt;=Summary!$B$3,L42&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -2285,7 +2479,7 @@
         <v>doc_09-R2</v>
       </c>
       <c r="B43" s="10" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C43" s="10" t="n">
         <v>2</v>
@@ -2296,13 +2490,16 @@
       <c r="G43" s="11"/>
       <c r="H43" s="11"/>
       <c r="I43" s="11"/>
-      <c r="J43" s="9"/>
-      <c r="K43" s="8" t="str">
-        <f aca="false">IF(COUNT(E43:H43)=4,AVERAGE(E43:H43),"")</f>
-        <v/>
-      </c>
-      <c r="L43" s="8" t="str">
-        <f aca="false">IF(K43="","",IF(AND(K43&gt;=Summary!$B$3,I43&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J43" s="11"/>
+      <c r="K43" s="11"/>
+      <c r="L43" s="11"/>
+      <c r="M43" s="9"/>
+      <c r="N43" s="8" t="str">
+        <f aca="false">IF(COUNT(H43:K43)=4,AVERAGE(H43:K43),"")</f>
+        <v/>
+      </c>
+      <c r="O43" s="8" t="str">
+        <f aca="false">IF(N43="","",IF(AND(N43&gt;=Summary!$B$3,L43&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -2312,7 +2509,7 @@
         <v>doc_09-R3</v>
       </c>
       <c r="B44" s="10" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C44" s="10" t="n">
         <v>3</v>
@@ -2323,13 +2520,16 @@
       <c r="G44" s="11"/>
       <c r="H44" s="11"/>
       <c r="I44" s="11"/>
-      <c r="J44" s="9"/>
-      <c r="K44" s="8" t="str">
-        <f aca="false">IF(COUNT(E44:H44)=4,AVERAGE(E44:H44),"")</f>
-        <v/>
-      </c>
-      <c r="L44" s="8" t="str">
-        <f aca="false">IF(K44="","",IF(AND(K44&gt;=Summary!$B$3,I44&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J44" s="11"/>
+      <c r="K44" s="11"/>
+      <c r="L44" s="11"/>
+      <c r="M44" s="9"/>
+      <c r="N44" s="8" t="str">
+        <f aca="false">IF(COUNT(H44:K44)=4,AVERAGE(H44:K44),"")</f>
+        <v/>
+      </c>
+      <c r="O44" s="8" t="str">
+        <f aca="false">IF(N44="","",IF(AND(N44&gt;=Summary!$B$3,L44&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -2339,7 +2539,7 @@
         <v>doc_09-R4</v>
       </c>
       <c r="B45" s="10" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C45" s="10" t="n">
         <v>4</v>
@@ -2350,13 +2550,16 @@
       <c r="G45" s="11"/>
       <c r="H45" s="11"/>
       <c r="I45" s="11"/>
-      <c r="J45" s="9"/>
-      <c r="K45" s="8" t="str">
-        <f aca="false">IF(COUNT(E45:H45)=4,AVERAGE(E45:H45),"")</f>
-        <v/>
-      </c>
-      <c r="L45" s="8" t="str">
-        <f aca="false">IF(K45="","",IF(AND(K45&gt;=Summary!$B$3,I45&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J45" s="11"/>
+      <c r="K45" s="11"/>
+      <c r="L45" s="11"/>
+      <c r="M45" s="9"/>
+      <c r="N45" s="8" t="str">
+        <f aca="false">IF(COUNT(H45:K45)=4,AVERAGE(H45:K45),"")</f>
+        <v/>
+      </c>
+      <c r="O45" s="8" t="str">
+        <f aca="false">IF(N45="","",IF(AND(N45&gt;=Summary!$B$3,L45&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -2366,7 +2569,7 @@
         <v>doc_09-R5</v>
       </c>
       <c r="B46" s="10" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C46" s="10" t="n">
         <v>5</v>
@@ -2377,13 +2580,16 @@
       <c r="G46" s="11"/>
       <c r="H46" s="11"/>
       <c r="I46" s="11"/>
-      <c r="J46" s="9"/>
-      <c r="K46" s="8" t="str">
-        <f aca="false">IF(COUNT(E46:H46)=4,AVERAGE(E46:H46),"")</f>
-        <v/>
-      </c>
-      <c r="L46" s="8" t="str">
-        <f aca="false">IF(K46="","",IF(AND(K46&gt;=Summary!$B$3,I46&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J46" s="11"/>
+      <c r="K46" s="11"/>
+      <c r="L46" s="11"/>
+      <c r="M46" s="9"/>
+      <c r="N46" s="8" t="str">
+        <f aca="false">IF(COUNT(H46:K46)=4,AVERAGE(H46:K46),"")</f>
+        <v/>
+      </c>
+      <c r="O46" s="8" t="str">
+        <f aca="false">IF(N46="","",IF(AND(N46&gt;=Summary!$B$3,L46&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -2393,7 +2599,7 @@
         <v>doc_10-R1</v>
       </c>
       <c r="B47" s="10" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C47" s="10" t="n">
         <v>1</v>
@@ -2404,13 +2610,16 @@
       <c r="G47" s="11"/>
       <c r="H47" s="11"/>
       <c r="I47" s="11"/>
-      <c r="J47" s="9"/>
-      <c r="K47" s="8" t="str">
-        <f aca="false">IF(COUNT(E47:H47)=4,AVERAGE(E47:H47),"")</f>
-        <v/>
-      </c>
-      <c r="L47" s="8" t="str">
-        <f aca="false">IF(K47="","",IF(AND(K47&gt;=Summary!$B$3,I47&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J47" s="11"/>
+      <c r="K47" s="11"/>
+      <c r="L47" s="11"/>
+      <c r="M47" s="9"/>
+      <c r="N47" s="8" t="str">
+        <f aca="false">IF(COUNT(H47:K47)=4,AVERAGE(H47:K47),"")</f>
+        <v/>
+      </c>
+      <c r="O47" s="8" t="str">
+        <f aca="false">IF(N47="","",IF(AND(N47&gt;=Summary!$B$3,L47&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -2420,7 +2629,7 @@
         <v>doc_10-R2</v>
       </c>
       <c r="B48" s="10" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C48" s="10" t="n">
         <v>2</v>
@@ -2431,13 +2640,16 @@
       <c r="G48" s="11"/>
       <c r="H48" s="11"/>
       <c r="I48" s="11"/>
-      <c r="J48" s="9"/>
-      <c r="K48" s="8" t="str">
-        <f aca="false">IF(COUNT(E48:H48)=4,AVERAGE(E48:H48),"")</f>
-        <v/>
-      </c>
-      <c r="L48" s="8" t="str">
-        <f aca="false">IF(K48="","",IF(AND(K48&gt;=Summary!$B$3,I48&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J48" s="11"/>
+      <c r="K48" s="11"/>
+      <c r="L48" s="11"/>
+      <c r="M48" s="9"/>
+      <c r="N48" s="8" t="str">
+        <f aca="false">IF(COUNT(H48:K48)=4,AVERAGE(H48:K48),"")</f>
+        <v/>
+      </c>
+      <c r="O48" s="8" t="str">
+        <f aca="false">IF(N48="","",IF(AND(N48&gt;=Summary!$B$3,L48&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -2447,7 +2659,7 @@
         <v>doc_10-R3</v>
       </c>
       <c r="B49" s="10" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C49" s="10" t="n">
         <v>3</v>
@@ -2458,13 +2670,16 @@
       <c r="G49" s="11"/>
       <c r="H49" s="11"/>
       <c r="I49" s="11"/>
-      <c r="J49" s="9"/>
-      <c r="K49" s="8" t="str">
-        <f aca="false">IF(COUNT(E49:H49)=4,AVERAGE(E49:H49),"")</f>
-        <v/>
-      </c>
-      <c r="L49" s="8" t="str">
-        <f aca="false">IF(K49="","",IF(AND(K49&gt;=Summary!$B$3,I49&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J49" s="11"/>
+      <c r="K49" s="11"/>
+      <c r="L49" s="11"/>
+      <c r="M49" s="9"/>
+      <c r="N49" s="8" t="str">
+        <f aca="false">IF(COUNT(H49:K49)=4,AVERAGE(H49:K49),"")</f>
+        <v/>
+      </c>
+      <c r="O49" s="8" t="str">
+        <f aca="false">IF(N49="","",IF(AND(N49&gt;=Summary!$B$3,L49&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -2474,7 +2689,7 @@
         <v>doc_10-R4</v>
       </c>
       <c r="B50" s="10" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C50" s="10" t="n">
         <v>4</v>
@@ -2485,13 +2700,16 @@
       <c r="G50" s="11"/>
       <c r="H50" s="11"/>
       <c r="I50" s="11"/>
-      <c r="J50" s="9"/>
-      <c r="K50" s="8" t="str">
-        <f aca="false">IF(COUNT(E50:H50)=4,AVERAGE(E50:H50),"")</f>
-        <v/>
-      </c>
-      <c r="L50" s="8" t="str">
-        <f aca="false">IF(K50="","",IF(AND(K50&gt;=Summary!$B$3,I50&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J50" s="11"/>
+      <c r="K50" s="11"/>
+      <c r="L50" s="11"/>
+      <c r="M50" s="9"/>
+      <c r="N50" s="8" t="str">
+        <f aca="false">IF(COUNT(H50:K50)=4,AVERAGE(H50:K50),"")</f>
+        <v/>
+      </c>
+      <c r="O50" s="8" t="str">
+        <f aca="false">IF(N50="","",IF(AND(N50&gt;=Summary!$B$3,L50&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -2501,7 +2719,7 @@
         <v>doc_10-R5</v>
       </c>
       <c r="B51" s="10" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C51" s="10" t="n">
         <v>5</v>
@@ -2512,13 +2730,16 @@
       <c r="G51" s="11"/>
       <c r="H51" s="11"/>
       <c r="I51" s="11"/>
-      <c r="J51" s="9"/>
-      <c r="K51" s="8" t="str">
-        <f aca="false">IF(COUNT(E51:H51)=4,AVERAGE(E51:H51),"")</f>
-        <v/>
-      </c>
-      <c r="L51" s="8" t="str">
-        <f aca="false">IF(K51="","",IF(AND(K51&gt;=Summary!$B$3,I51&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J51" s="11"/>
+      <c r="K51" s="11"/>
+      <c r="L51" s="11"/>
+      <c r="M51" s="9"/>
+      <c r="N51" s="8" t="str">
+        <f aca="false">IF(COUNT(H51:K51)=4,AVERAGE(H51:K51),"")</f>
+        <v/>
+      </c>
+      <c r="O51" s="8" t="str">
+        <f aca="false">IF(N51="","",IF(AND(N51&gt;=Summary!$B$3,L51&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -2528,7 +2749,7 @@
         <v>doc_11-R1</v>
       </c>
       <c r="B52" s="10" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C52" s="10" t="n">
         <v>1</v>
@@ -2539,13 +2760,16 @@
       <c r="G52" s="11"/>
       <c r="H52" s="11"/>
       <c r="I52" s="11"/>
-      <c r="J52" s="9"/>
-      <c r="K52" s="8" t="str">
-        <f aca="false">IF(COUNT(E52:H52)=4,AVERAGE(E52:H52),"")</f>
-        <v/>
-      </c>
-      <c r="L52" s="8" t="str">
-        <f aca="false">IF(K52="","",IF(AND(K52&gt;=Summary!$B$3,I52&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J52" s="11"/>
+      <c r="K52" s="11"/>
+      <c r="L52" s="11"/>
+      <c r="M52" s="9"/>
+      <c r="N52" s="8" t="str">
+        <f aca="false">IF(COUNT(H52:K52)=4,AVERAGE(H52:K52),"")</f>
+        <v/>
+      </c>
+      <c r="O52" s="8" t="str">
+        <f aca="false">IF(N52="","",IF(AND(N52&gt;=Summary!$B$3,L52&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -2555,7 +2779,7 @@
         <v>doc_11-R2</v>
       </c>
       <c r="B53" s="10" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C53" s="10" t="n">
         <v>2</v>
@@ -2566,13 +2790,16 @@
       <c r="G53" s="11"/>
       <c r="H53" s="11"/>
       <c r="I53" s="11"/>
-      <c r="J53" s="9"/>
-      <c r="K53" s="8" t="str">
-        <f aca="false">IF(COUNT(E53:H53)=4,AVERAGE(E53:H53),"")</f>
-        <v/>
-      </c>
-      <c r="L53" s="8" t="str">
-        <f aca="false">IF(K53="","",IF(AND(K53&gt;=Summary!$B$3,I53&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J53" s="11"/>
+      <c r="K53" s="11"/>
+      <c r="L53" s="11"/>
+      <c r="M53" s="9"/>
+      <c r="N53" s="8" t="str">
+        <f aca="false">IF(COUNT(H53:K53)=4,AVERAGE(H53:K53),"")</f>
+        <v/>
+      </c>
+      <c r="O53" s="8" t="str">
+        <f aca="false">IF(N53="","",IF(AND(N53&gt;=Summary!$B$3,L53&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -2582,7 +2809,7 @@
         <v>doc_11-R3</v>
       </c>
       <c r="B54" s="10" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C54" s="10" t="n">
         <v>3</v>
@@ -2593,13 +2820,16 @@
       <c r="G54" s="11"/>
       <c r="H54" s="11"/>
       <c r="I54" s="11"/>
-      <c r="J54" s="9"/>
-      <c r="K54" s="8" t="str">
-        <f aca="false">IF(COUNT(E54:H54)=4,AVERAGE(E54:H54),"")</f>
-        <v/>
-      </c>
-      <c r="L54" s="8" t="str">
-        <f aca="false">IF(K54="","",IF(AND(K54&gt;=Summary!$B$3,I54&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J54" s="11"/>
+      <c r="K54" s="11"/>
+      <c r="L54" s="11"/>
+      <c r="M54" s="9"/>
+      <c r="N54" s="8" t="str">
+        <f aca="false">IF(COUNT(H54:K54)=4,AVERAGE(H54:K54),"")</f>
+        <v/>
+      </c>
+      <c r="O54" s="8" t="str">
+        <f aca="false">IF(N54="","",IF(AND(N54&gt;=Summary!$B$3,L54&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -2609,7 +2839,7 @@
         <v>doc_11-R4</v>
       </c>
       <c r="B55" s="10" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C55" s="10" t="n">
         <v>4</v>
@@ -2620,13 +2850,16 @@
       <c r="G55" s="11"/>
       <c r="H55" s="11"/>
       <c r="I55" s="11"/>
-      <c r="J55" s="9"/>
-      <c r="K55" s="8" t="str">
-        <f aca="false">IF(COUNT(E55:H55)=4,AVERAGE(E55:H55),"")</f>
-        <v/>
-      </c>
-      <c r="L55" s="8" t="str">
-        <f aca="false">IF(K55="","",IF(AND(K55&gt;=Summary!$B$3,I55&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J55" s="11"/>
+      <c r="K55" s="11"/>
+      <c r="L55" s="11"/>
+      <c r="M55" s="9"/>
+      <c r="N55" s="8" t="str">
+        <f aca="false">IF(COUNT(H55:K55)=4,AVERAGE(H55:K55),"")</f>
+        <v/>
+      </c>
+      <c r="O55" s="8" t="str">
+        <f aca="false">IF(N55="","",IF(AND(N55&gt;=Summary!$B$3,L55&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -2636,7 +2869,7 @@
         <v>doc_11-R5</v>
       </c>
       <c r="B56" s="10" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C56" s="10" t="n">
         <v>5</v>
@@ -2647,13 +2880,16 @@
       <c r="G56" s="11"/>
       <c r="H56" s="11"/>
       <c r="I56" s="11"/>
-      <c r="J56" s="9"/>
-      <c r="K56" s="8" t="str">
-        <f aca="false">IF(COUNT(E56:H56)=4,AVERAGE(E56:H56),"")</f>
-        <v/>
-      </c>
-      <c r="L56" s="8" t="str">
-        <f aca="false">IF(K56="","",IF(AND(K56&gt;=Summary!$B$3,I56&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J56" s="11"/>
+      <c r="K56" s="11"/>
+      <c r="L56" s="11"/>
+      <c r="M56" s="9"/>
+      <c r="N56" s="8" t="str">
+        <f aca="false">IF(COUNT(H56:K56)=4,AVERAGE(H56:K56),"")</f>
+        <v/>
+      </c>
+      <c r="O56" s="8" t="str">
+        <f aca="false">IF(N56="","",IF(AND(N56&gt;=Summary!$B$3,L56&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -2663,7 +2899,7 @@
         <v>doc_12-R1</v>
       </c>
       <c r="B57" s="10" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C57" s="10" t="n">
         <v>1</v>
@@ -2674,13 +2910,16 @@
       <c r="G57" s="11"/>
       <c r="H57" s="11"/>
       <c r="I57" s="11"/>
-      <c r="J57" s="9"/>
-      <c r="K57" s="8" t="str">
-        <f aca="false">IF(COUNT(E57:H57)=4,AVERAGE(E57:H57),"")</f>
-        <v/>
-      </c>
-      <c r="L57" s="8" t="str">
-        <f aca="false">IF(K57="","",IF(AND(K57&gt;=Summary!$B$3,I57&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J57" s="11"/>
+      <c r="K57" s="11"/>
+      <c r="L57" s="11"/>
+      <c r="M57" s="9"/>
+      <c r="N57" s="8" t="str">
+        <f aca="false">IF(COUNT(H57:K57)=4,AVERAGE(H57:K57),"")</f>
+        <v/>
+      </c>
+      <c r="O57" s="8" t="str">
+        <f aca="false">IF(N57="","",IF(AND(N57&gt;=Summary!$B$3,L57&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -2690,7 +2929,7 @@
         <v>doc_12-R2</v>
       </c>
       <c r="B58" s="10" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C58" s="10" t="n">
         <v>2</v>
@@ -2701,13 +2940,16 @@
       <c r="G58" s="11"/>
       <c r="H58" s="11"/>
       <c r="I58" s="11"/>
-      <c r="J58" s="9"/>
-      <c r="K58" s="8" t="str">
-        <f aca="false">IF(COUNT(E58:H58)=4,AVERAGE(E58:H58),"")</f>
-        <v/>
-      </c>
-      <c r="L58" s="8" t="str">
-        <f aca="false">IF(K58="","",IF(AND(K58&gt;=Summary!$B$3,I58&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J58" s="11"/>
+      <c r="K58" s="11"/>
+      <c r="L58" s="11"/>
+      <c r="M58" s="9"/>
+      <c r="N58" s="8" t="str">
+        <f aca="false">IF(COUNT(H58:K58)=4,AVERAGE(H58:K58),"")</f>
+        <v/>
+      </c>
+      <c r="O58" s="8" t="str">
+        <f aca="false">IF(N58="","",IF(AND(N58&gt;=Summary!$B$3,L58&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -2717,7 +2959,7 @@
         <v>doc_12-R3</v>
       </c>
       <c r="B59" s="10" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C59" s="10" t="n">
         <v>3</v>
@@ -2728,13 +2970,16 @@
       <c r="G59" s="11"/>
       <c r="H59" s="11"/>
       <c r="I59" s="11"/>
-      <c r="J59" s="9"/>
-      <c r="K59" s="8" t="str">
-        <f aca="false">IF(COUNT(E59:H59)=4,AVERAGE(E59:H59),"")</f>
-        <v/>
-      </c>
-      <c r="L59" s="8" t="str">
-        <f aca="false">IF(K59="","",IF(AND(K59&gt;=Summary!$B$3,I59&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J59" s="11"/>
+      <c r="K59" s="11"/>
+      <c r="L59" s="11"/>
+      <c r="M59" s="9"/>
+      <c r="N59" s="8" t="str">
+        <f aca="false">IF(COUNT(H59:K59)=4,AVERAGE(H59:K59),"")</f>
+        <v/>
+      </c>
+      <c r="O59" s="8" t="str">
+        <f aca="false">IF(N59="","",IF(AND(N59&gt;=Summary!$B$3,L59&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -2744,7 +2989,7 @@
         <v>doc_12-R4</v>
       </c>
       <c r="B60" s="10" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C60" s="10" t="n">
         <v>4</v>
@@ -2755,13 +3000,16 @@
       <c r="G60" s="11"/>
       <c r="H60" s="11"/>
       <c r="I60" s="11"/>
-      <c r="J60" s="9"/>
-      <c r="K60" s="8" t="str">
-        <f aca="false">IF(COUNT(E60:H60)=4,AVERAGE(E60:H60),"")</f>
-        <v/>
-      </c>
-      <c r="L60" s="8" t="str">
-        <f aca="false">IF(K60="","",IF(AND(K60&gt;=Summary!$B$3,I60&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J60" s="11"/>
+      <c r="K60" s="11"/>
+      <c r="L60" s="11"/>
+      <c r="M60" s="9"/>
+      <c r="N60" s="8" t="str">
+        <f aca="false">IF(COUNT(H60:K60)=4,AVERAGE(H60:K60),"")</f>
+        <v/>
+      </c>
+      <c r="O60" s="8" t="str">
+        <f aca="false">IF(N60="","",IF(AND(N60&gt;=Summary!$B$3,L60&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -2771,7 +3019,7 @@
         <v>doc_12-R5</v>
       </c>
       <c r="B61" s="10" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C61" s="10" t="n">
         <v>5</v>
@@ -2782,13 +3030,16 @@
       <c r="G61" s="11"/>
       <c r="H61" s="11"/>
       <c r="I61" s="11"/>
-      <c r="J61" s="9"/>
-      <c r="K61" s="8" t="str">
-        <f aca="false">IF(COUNT(E61:H61)=4,AVERAGE(E61:H61),"")</f>
-        <v/>
-      </c>
-      <c r="L61" s="8" t="str">
-        <f aca="false">IF(K61="","",IF(AND(K61&gt;=Summary!$B$3,I61&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J61" s="11"/>
+      <c r="K61" s="11"/>
+      <c r="L61" s="11"/>
+      <c r="M61" s="9"/>
+      <c r="N61" s="8" t="str">
+        <f aca="false">IF(COUNT(H61:K61)=4,AVERAGE(H61:K61),"")</f>
+        <v/>
+      </c>
+      <c r="O61" s="8" t="str">
+        <f aca="false">IF(N61="","",IF(AND(N61&gt;=Summary!$B$3,L61&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -2798,7 +3049,7 @@
         <v>doc_13-R1</v>
       </c>
       <c r="B62" s="10" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C62" s="10" t="n">
         <v>1</v>
@@ -2809,13 +3060,16 @@
       <c r="G62" s="11"/>
       <c r="H62" s="11"/>
       <c r="I62" s="11"/>
-      <c r="J62" s="9"/>
-      <c r="K62" s="8" t="str">
-        <f aca="false">IF(COUNT(E62:H62)=4,AVERAGE(E62:H62),"")</f>
-        <v/>
-      </c>
-      <c r="L62" s="8" t="str">
-        <f aca="false">IF(K62="","",IF(AND(K62&gt;=Summary!$B$3,I62&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J62" s="11"/>
+      <c r="K62" s="11"/>
+      <c r="L62" s="11"/>
+      <c r="M62" s="9"/>
+      <c r="N62" s="8" t="str">
+        <f aca="false">IF(COUNT(H62:K62)=4,AVERAGE(H62:K62),"")</f>
+        <v/>
+      </c>
+      <c r="O62" s="8" t="str">
+        <f aca="false">IF(N62="","",IF(AND(N62&gt;=Summary!$B$3,L62&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -2825,7 +3079,7 @@
         <v>doc_13-R2</v>
       </c>
       <c r="B63" s="10" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C63" s="10" t="n">
         <v>2</v>
@@ -2836,13 +3090,16 @@
       <c r="G63" s="11"/>
       <c r="H63" s="11"/>
       <c r="I63" s="11"/>
-      <c r="J63" s="9"/>
-      <c r="K63" s="8" t="str">
-        <f aca="false">IF(COUNT(E63:H63)=4,AVERAGE(E63:H63),"")</f>
-        <v/>
-      </c>
-      <c r="L63" s="8" t="str">
-        <f aca="false">IF(K63="","",IF(AND(K63&gt;=Summary!$B$3,I63&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J63" s="11"/>
+      <c r="K63" s="11"/>
+      <c r="L63" s="11"/>
+      <c r="M63" s="9"/>
+      <c r="N63" s="8" t="str">
+        <f aca="false">IF(COUNT(H63:K63)=4,AVERAGE(H63:K63),"")</f>
+        <v/>
+      </c>
+      <c r="O63" s="8" t="str">
+        <f aca="false">IF(N63="","",IF(AND(N63&gt;=Summary!$B$3,L63&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -2852,7 +3109,7 @@
         <v>doc_13-R3</v>
       </c>
       <c r="B64" s="10" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C64" s="10" t="n">
         <v>3</v>
@@ -2863,13 +3120,16 @@
       <c r="G64" s="11"/>
       <c r="H64" s="11"/>
       <c r="I64" s="11"/>
-      <c r="J64" s="9"/>
-      <c r="K64" s="8" t="str">
-        <f aca="false">IF(COUNT(E64:H64)=4,AVERAGE(E64:H64),"")</f>
-        <v/>
-      </c>
-      <c r="L64" s="8" t="str">
-        <f aca="false">IF(K64="","",IF(AND(K64&gt;=Summary!$B$3,I64&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J64" s="11"/>
+      <c r="K64" s="11"/>
+      <c r="L64" s="11"/>
+      <c r="M64" s="9"/>
+      <c r="N64" s="8" t="str">
+        <f aca="false">IF(COUNT(H64:K64)=4,AVERAGE(H64:K64),"")</f>
+        <v/>
+      </c>
+      <c r="O64" s="8" t="str">
+        <f aca="false">IF(N64="","",IF(AND(N64&gt;=Summary!$B$3,L64&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -2879,7 +3139,7 @@
         <v>doc_13-R4</v>
       </c>
       <c r="B65" s="10" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C65" s="10" t="n">
         <v>4</v>
@@ -2890,13 +3150,16 @@
       <c r="G65" s="11"/>
       <c r="H65" s="11"/>
       <c r="I65" s="11"/>
-      <c r="J65" s="9"/>
-      <c r="K65" s="8" t="str">
-        <f aca="false">IF(COUNT(E65:H65)=4,AVERAGE(E65:H65),"")</f>
-        <v/>
-      </c>
-      <c r="L65" s="8" t="str">
-        <f aca="false">IF(K65="","",IF(AND(K65&gt;=Summary!$B$3,I65&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J65" s="11"/>
+      <c r="K65" s="11"/>
+      <c r="L65" s="11"/>
+      <c r="M65" s="9"/>
+      <c r="N65" s="8" t="str">
+        <f aca="false">IF(COUNT(H65:K65)=4,AVERAGE(H65:K65),"")</f>
+        <v/>
+      </c>
+      <c r="O65" s="8" t="str">
+        <f aca="false">IF(N65="","",IF(AND(N65&gt;=Summary!$B$3,L65&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -2906,7 +3169,7 @@
         <v>doc_13-R5</v>
       </c>
       <c r="B66" s="10" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C66" s="10" t="n">
         <v>5</v>
@@ -2917,13 +3180,16 @@
       <c r="G66" s="11"/>
       <c r="H66" s="11"/>
       <c r="I66" s="11"/>
-      <c r="J66" s="9"/>
-      <c r="K66" s="8" t="str">
-        <f aca="false">IF(COUNT(E66:H66)=4,AVERAGE(E66:H66),"")</f>
-        <v/>
-      </c>
-      <c r="L66" s="8" t="str">
-        <f aca="false">IF(K66="","",IF(AND(K66&gt;=Summary!$B$3,I66&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J66" s="11"/>
+      <c r="K66" s="11"/>
+      <c r="L66" s="11"/>
+      <c r="M66" s="9"/>
+      <c r="N66" s="8" t="str">
+        <f aca="false">IF(COUNT(H66:K66)=4,AVERAGE(H66:K66),"")</f>
+        <v/>
+      </c>
+      <c r="O66" s="8" t="str">
+        <f aca="false">IF(N66="","",IF(AND(N66&gt;=Summary!$B$3,L66&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -2933,7 +3199,7 @@
         <v>doc_14-R1</v>
       </c>
       <c r="B67" s="10" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C67" s="10" t="n">
         <v>1</v>
@@ -2944,13 +3210,16 @@
       <c r="G67" s="11"/>
       <c r="H67" s="11"/>
       <c r="I67" s="11"/>
-      <c r="J67" s="9"/>
-      <c r="K67" s="8" t="str">
-        <f aca="false">IF(COUNT(E67:H67)=4,AVERAGE(E67:H67),"")</f>
-        <v/>
-      </c>
-      <c r="L67" s="8" t="str">
-        <f aca="false">IF(K67="","",IF(AND(K67&gt;=Summary!$B$3,I67&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J67" s="11"/>
+      <c r="K67" s="11"/>
+      <c r="L67" s="11"/>
+      <c r="M67" s="9"/>
+      <c r="N67" s="8" t="str">
+        <f aca="false">IF(COUNT(H67:K67)=4,AVERAGE(H67:K67),"")</f>
+        <v/>
+      </c>
+      <c r="O67" s="8" t="str">
+        <f aca="false">IF(N67="","",IF(AND(N67&gt;=Summary!$B$3,L67&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -2960,7 +3229,7 @@
         <v>doc_14-R2</v>
       </c>
       <c r="B68" s="10" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C68" s="10" t="n">
         <v>2</v>
@@ -2971,13 +3240,16 @@
       <c r="G68" s="11"/>
       <c r="H68" s="11"/>
       <c r="I68" s="11"/>
-      <c r="J68" s="9"/>
-      <c r="K68" s="8" t="str">
-        <f aca="false">IF(COUNT(E68:H68)=4,AVERAGE(E68:H68),"")</f>
-        <v/>
-      </c>
-      <c r="L68" s="8" t="str">
-        <f aca="false">IF(K68="","",IF(AND(K68&gt;=Summary!$B$3,I68&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J68" s="11"/>
+      <c r="K68" s="11"/>
+      <c r="L68" s="11"/>
+      <c r="M68" s="9"/>
+      <c r="N68" s="8" t="str">
+        <f aca="false">IF(COUNT(H68:K68)=4,AVERAGE(H68:K68),"")</f>
+        <v/>
+      </c>
+      <c r="O68" s="8" t="str">
+        <f aca="false">IF(N68="","",IF(AND(N68&gt;=Summary!$B$3,L68&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -2987,7 +3259,7 @@
         <v>doc_14-R3</v>
       </c>
       <c r="B69" s="10" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C69" s="10" t="n">
         <v>3</v>
@@ -2998,13 +3270,16 @@
       <c r="G69" s="11"/>
       <c r="H69" s="11"/>
       <c r="I69" s="11"/>
-      <c r="J69" s="9"/>
-      <c r="K69" s="8" t="str">
-        <f aca="false">IF(COUNT(E69:H69)=4,AVERAGE(E69:H69),"")</f>
-        <v/>
-      </c>
-      <c r="L69" s="8" t="str">
-        <f aca="false">IF(K69="","",IF(AND(K69&gt;=Summary!$B$3,I69&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J69" s="11"/>
+      <c r="K69" s="11"/>
+      <c r="L69" s="11"/>
+      <c r="M69" s="9"/>
+      <c r="N69" s="8" t="str">
+        <f aca="false">IF(COUNT(H69:K69)=4,AVERAGE(H69:K69),"")</f>
+        <v/>
+      </c>
+      <c r="O69" s="8" t="str">
+        <f aca="false">IF(N69="","",IF(AND(N69&gt;=Summary!$B$3,L69&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -3014,7 +3289,7 @@
         <v>doc_14-R4</v>
       </c>
       <c r="B70" s="10" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C70" s="10" t="n">
         <v>4</v>
@@ -3025,13 +3300,16 @@
       <c r="G70" s="11"/>
       <c r="H70" s="11"/>
       <c r="I70" s="11"/>
-      <c r="J70" s="9"/>
-      <c r="K70" s="8" t="str">
-        <f aca="false">IF(COUNT(E70:H70)=4,AVERAGE(E70:H70),"")</f>
-        <v/>
-      </c>
-      <c r="L70" s="8" t="str">
-        <f aca="false">IF(K70="","",IF(AND(K70&gt;=Summary!$B$3,I70&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J70" s="11"/>
+      <c r="K70" s="11"/>
+      <c r="L70" s="11"/>
+      <c r="M70" s="9"/>
+      <c r="N70" s="8" t="str">
+        <f aca="false">IF(COUNT(H70:K70)=4,AVERAGE(H70:K70),"")</f>
+        <v/>
+      </c>
+      <c r="O70" s="8" t="str">
+        <f aca="false">IF(N70="","",IF(AND(N70&gt;=Summary!$B$3,L70&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -3041,7 +3319,7 @@
         <v>doc_14-R5</v>
       </c>
       <c r="B71" s="10" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C71" s="10" t="n">
         <v>5</v>
@@ -3052,13 +3330,16 @@
       <c r="G71" s="11"/>
       <c r="H71" s="11"/>
       <c r="I71" s="11"/>
-      <c r="J71" s="9"/>
-      <c r="K71" s="8" t="str">
-        <f aca="false">IF(COUNT(E71:H71)=4,AVERAGE(E71:H71),"")</f>
-        <v/>
-      </c>
-      <c r="L71" s="8" t="str">
-        <f aca="false">IF(K71="","",IF(AND(K71&gt;=Summary!$B$3,I71&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J71" s="11"/>
+      <c r="K71" s="11"/>
+      <c r="L71" s="11"/>
+      <c r="M71" s="9"/>
+      <c r="N71" s="8" t="str">
+        <f aca="false">IF(COUNT(H71:K71)=4,AVERAGE(H71:K71),"")</f>
+        <v/>
+      </c>
+      <c r="O71" s="8" t="str">
+        <f aca="false">IF(N71="","",IF(AND(N71&gt;=Summary!$B$3,L71&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -3068,7 +3349,7 @@
         <v>doc_15-R1</v>
       </c>
       <c r="B72" s="10" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C72" s="10" t="n">
         <v>1</v>
@@ -3079,13 +3360,16 @@
       <c r="G72" s="11"/>
       <c r="H72" s="11"/>
       <c r="I72" s="11"/>
-      <c r="J72" s="9"/>
-      <c r="K72" s="8" t="str">
-        <f aca="false">IF(COUNT(E72:H72)=4,AVERAGE(E72:H72),"")</f>
-        <v/>
-      </c>
-      <c r="L72" s="8" t="str">
-        <f aca="false">IF(K72="","",IF(AND(K72&gt;=Summary!$B$3,I72&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J72" s="11"/>
+      <c r="K72" s="11"/>
+      <c r="L72" s="11"/>
+      <c r="M72" s="9"/>
+      <c r="N72" s="8" t="str">
+        <f aca="false">IF(COUNT(H72:K72)=4,AVERAGE(H72:K72),"")</f>
+        <v/>
+      </c>
+      <c r="O72" s="8" t="str">
+        <f aca="false">IF(N72="","",IF(AND(N72&gt;=Summary!$B$3,L72&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -3095,7 +3379,7 @@
         <v>doc_15-R2</v>
       </c>
       <c r="B73" s="10" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C73" s="10" t="n">
         <v>2</v>
@@ -3106,13 +3390,16 @@
       <c r="G73" s="11"/>
       <c r="H73" s="11"/>
       <c r="I73" s="11"/>
-      <c r="J73" s="9"/>
-      <c r="K73" s="8" t="str">
-        <f aca="false">IF(COUNT(E73:H73)=4,AVERAGE(E73:H73),"")</f>
-        <v/>
-      </c>
-      <c r="L73" s="8" t="str">
-        <f aca="false">IF(K73="","",IF(AND(K73&gt;=Summary!$B$3,I73&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J73" s="11"/>
+      <c r="K73" s="11"/>
+      <c r="L73" s="11"/>
+      <c r="M73" s="9"/>
+      <c r="N73" s="8" t="str">
+        <f aca="false">IF(COUNT(H73:K73)=4,AVERAGE(H73:K73),"")</f>
+        <v/>
+      </c>
+      <c r="O73" s="8" t="str">
+        <f aca="false">IF(N73="","",IF(AND(N73&gt;=Summary!$B$3,L73&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -3122,7 +3409,7 @@
         <v>doc_15-R3</v>
       </c>
       <c r="B74" s="10" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C74" s="10" t="n">
         <v>3</v>
@@ -3133,13 +3420,16 @@
       <c r="G74" s="11"/>
       <c r="H74" s="11"/>
       <c r="I74" s="11"/>
-      <c r="J74" s="9"/>
-      <c r="K74" s="8" t="str">
-        <f aca="false">IF(COUNT(E74:H74)=4,AVERAGE(E74:H74),"")</f>
-        <v/>
-      </c>
-      <c r="L74" s="8" t="str">
-        <f aca="false">IF(K74="","",IF(AND(K74&gt;=Summary!$B$3,I74&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J74" s="11"/>
+      <c r="K74" s="11"/>
+      <c r="L74" s="11"/>
+      <c r="M74" s="9"/>
+      <c r="N74" s="8" t="str">
+        <f aca="false">IF(COUNT(H74:K74)=4,AVERAGE(H74:K74),"")</f>
+        <v/>
+      </c>
+      <c r="O74" s="8" t="str">
+        <f aca="false">IF(N74="","",IF(AND(N74&gt;=Summary!$B$3,L74&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -3149,7 +3439,7 @@
         <v>doc_15-R4</v>
       </c>
       <c r="B75" s="10" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C75" s="10" t="n">
         <v>4</v>
@@ -3160,13 +3450,16 @@
       <c r="G75" s="11"/>
       <c r="H75" s="11"/>
       <c r="I75" s="11"/>
-      <c r="J75" s="9"/>
-      <c r="K75" s="8" t="str">
-        <f aca="false">IF(COUNT(E75:H75)=4,AVERAGE(E75:H75),"")</f>
-        <v/>
-      </c>
-      <c r="L75" s="8" t="str">
-        <f aca="false">IF(K75="","",IF(AND(K75&gt;=Summary!$B$3,I75&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J75" s="11"/>
+      <c r="K75" s="11"/>
+      <c r="L75" s="11"/>
+      <c r="M75" s="9"/>
+      <c r="N75" s="8" t="str">
+        <f aca="false">IF(COUNT(H75:K75)=4,AVERAGE(H75:K75),"")</f>
+        <v/>
+      </c>
+      <c r="O75" s="8" t="str">
+        <f aca="false">IF(N75="","",IF(AND(N75&gt;=Summary!$B$3,L75&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -3176,7 +3469,7 @@
         <v>doc_15-R5</v>
       </c>
       <c r="B76" s="10" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C76" s="10" t="n">
         <v>5</v>
@@ -3187,18 +3480,21 @@
       <c r="G76" s="11"/>
       <c r="H76" s="11"/>
       <c r="I76" s="11"/>
-      <c r="J76" s="9"/>
-      <c r="K76" s="8" t="str">
-        <f aca="false">IF(COUNT(E76:H76)=4,AVERAGE(E76:H76),"")</f>
-        <v/>
-      </c>
-      <c r="L76" s="8" t="str">
-        <f aca="false">IF(K76="","",IF(AND(K76&gt;=Summary!$B$3,I76&lt;=Summary!$B$4),"PASS","FAIL"))</f>
+      <c r="J76" s="11"/>
+      <c r="K76" s="11"/>
+      <c r="L76" s="11"/>
+      <c r="M76" s="9"/>
+      <c r="N76" s="8" t="str">
+        <f aca="false">IF(COUNT(H76:K76)=4,AVERAGE(H76:K76),"")</f>
+        <v/>
+      </c>
+      <c r="O76" s="8" t="str">
+        <f aca="false">IF(N76="","",IF(AND(N76&gt;=Summary!$B$3,L76&lt;=Summary!$B$4),"PASS","FAIL"))</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="4">
+  <dataValidations count="7">
     <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B2:B76" type="list">
       <formula1>"doc_01,doc_02,doc_03,doc_04,doc_05,doc_06,doc_07,doc_08,doc_09,doc_10,doc_11,doc_12,doc_13,doc_14,doc_15"</formula1>
       <formula2>0</formula2>
@@ -3207,11 +3503,23 @@
       <formula1>"1,2,3,4,5"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E2:H76" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E2:E76" type="list">
+      <formula1>"NONE,LIGHT,MODERATE,SEVERE,CRITICAL,EMERGENCY,SHUTDOWN"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" error="Enter a battery percentage between 0 and 100." errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F2:F76" type="whole">
+      <formula1>0</formula1>
+      <formula2>100</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G2:G76" type="list">
+      <formula1>"Charging,Discharging,Full,Not charging"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H2:K76" type="list">
       <formula1>"1,2,3,4,5"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I2:I76" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="L2:L76" type="list">
       <formula1>"0,1,2,3,4,5"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -3231,7 +3539,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:E57"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="48"/>
@@ -3240,64 +3548,64 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="12" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="B3" s="13" t="n">
         <v>3.5</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="B4" s="13" t="n">
         <v>0</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="B5" s="13" t="n">
         <v>0.8</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="B8" s="0" t="n">
-        <f aca="false">COUNT('Raw Scores'!K2:K76)</f>
+        <f aca="false">COUNT('Raw Scores'!N2:N76)</f>
         <v>0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="B9" s="0" t="n">
         <f aca="false">75-B8</f>
@@ -3306,66 +3614,66 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="B12" s="15" t="str">
-        <f aca="false">IF(B8=0,"",AVERAGE('Raw Scores'!K2:K76))</f>
+        <f aca="false">IF(B8=0,"",AVERAGE('Raw Scores'!N2:N76))</f>
         <v/>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="B13" s="15" t="str">
-        <f aca="false">IF(B8=0,"",MEDIAN('Raw Scores'!K2:K76))</f>
+        <f aca="false">IF(B8=0,"",MEDIAN('Raw Scores'!N2:N76))</f>
         <v/>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="B14" s="15" t="n">
-        <f aca="false">COUNTIF('Raw Scores'!L2:L76,"PASS")</f>
+        <f aca="false">COUNTIF('Raw Scores'!O2:O76,"PASS")</f>
         <v>0</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="B15" s="15" t="str">
-        <f aca="false">IF(B8=0,"",COUNTIF('Raw Scores'!L2:L76,"PASS")/B8)</f>
+        <f aca="false">IF(B8=0,"",COUNTIF('Raw Scores'!O2:O76,"PASS")/B8)</f>
         <v/>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="B16" s="15" t="n">
-        <f aca="false">COUNTIF('Raw Scores'!I2:I76,"&gt;0")</f>
+        <f aca="false">COUNTIF('Raw Scores'!L2:L76,"&gt;0")</f>
         <v>0</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="B17" s="15" t="str">
-        <f aca="false">IF(B8=0,"",COUNTIF('Raw Scores'!I2:I76,"&gt;0")/B8)</f>
+        <f aca="false">IF(B8=0,"",COUNTIF('Raw Scores'!L2:L76,"&gt;0")/B8)</f>
         <v/>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="B19" s="16" t="str">
         <f aca="false">IF(B8&lt;75,"INCOMPLETE",IF(AND(B16&gt;=B5,B18&lt;=1-B5),"MODEL RETAINED","MODEL NOT RETAINED - review"))</f>
@@ -3374,29 +3682,29 @@
     </row>
     <row r="20" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="17" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="0" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3404,19 +3712,19 @@
         <v>1</v>
       </c>
       <c r="B25" s="15" t="n">
-        <f aca="false">COUNTIF('Raw Scores'!E2:E76,1)</f>
+        <f aca="false">COUNTIF('Raw Scores'!H2:H76,1)</f>
         <v>0</v>
       </c>
       <c r="C25" s="15" t="n">
-        <f aca="false">COUNTIF('Raw Scores'!F2:F76,1)</f>
+        <f aca="false">COUNTIF('Raw Scores'!I2:I76,1)</f>
         <v>0</v>
       </c>
       <c r="D25" s="15" t="n">
-        <f aca="false">COUNTIF('Raw Scores'!G2:G76,1)</f>
+        <f aca="false">COUNTIF('Raw Scores'!J2:J76,1)</f>
         <v>0</v>
       </c>
       <c r="E25" s="15" t="n">
-        <f aca="false">COUNTIF('Raw Scores'!H2:H76,1)</f>
+        <f aca="false">COUNTIF('Raw Scores'!K2:K76,1)</f>
         <v>0</v>
       </c>
     </row>
@@ -3425,19 +3733,19 @@
         <v>2</v>
       </c>
       <c r="B26" s="15" t="n">
-        <f aca="false">COUNTIF('Raw Scores'!E2:E76,2)</f>
+        <f aca="false">COUNTIF('Raw Scores'!H2:H76,2)</f>
         <v>0</v>
       </c>
       <c r="C26" s="15" t="n">
-        <f aca="false">COUNTIF('Raw Scores'!F2:F76,2)</f>
+        <f aca="false">COUNTIF('Raw Scores'!I2:I76,2)</f>
         <v>0</v>
       </c>
       <c r="D26" s="15" t="n">
-        <f aca="false">COUNTIF('Raw Scores'!G2:G76,2)</f>
+        <f aca="false">COUNTIF('Raw Scores'!J2:J76,2)</f>
         <v>0</v>
       </c>
       <c r="E26" s="15" t="n">
-        <f aca="false">COUNTIF('Raw Scores'!H2:H76,2)</f>
+        <f aca="false">COUNTIF('Raw Scores'!K2:K76,2)</f>
         <v>0</v>
       </c>
     </row>
@@ -3446,19 +3754,19 @@
         <v>3</v>
       </c>
       <c r="B27" s="15" t="n">
-        <f aca="false">COUNTIF('Raw Scores'!E2:E76,3)</f>
+        <f aca="false">COUNTIF('Raw Scores'!H2:H76,3)</f>
         <v>0</v>
       </c>
       <c r="C27" s="15" t="n">
-        <f aca="false">COUNTIF('Raw Scores'!F2:F76,3)</f>
+        <f aca="false">COUNTIF('Raw Scores'!I2:I76,3)</f>
         <v>0</v>
       </c>
       <c r="D27" s="15" t="n">
-        <f aca="false">COUNTIF('Raw Scores'!G2:G76,3)</f>
+        <f aca="false">COUNTIF('Raw Scores'!J2:J76,3)</f>
         <v>0</v>
       </c>
       <c r="E27" s="15" t="n">
-        <f aca="false">COUNTIF('Raw Scores'!H2:H76,3)</f>
+        <f aca="false">COUNTIF('Raw Scores'!K2:K76,3)</f>
         <v>0</v>
       </c>
     </row>
@@ -3467,19 +3775,19 @@
         <v>4</v>
       </c>
       <c r="B28" s="15" t="n">
-        <f aca="false">COUNTIF('Raw Scores'!E2:E76,4)</f>
+        <f aca="false">COUNTIF('Raw Scores'!H2:H76,4)</f>
         <v>0</v>
       </c>
       <c r="C28" s="15" t="n">
-        <f aca="false">COUNTIF('Raw Scores'!F2:F76,4)</f>
+        <f aca="false">COUNTIF('Raw Scores'!I2:I76,4)</f>
         <v>0</v>
       </c>
       <c r="D28" s="15" t="n">
-        <f aca="false">COUNTIF('Raw Scores'!G2:G76,4)</f>
+        <f aca="false">COUNTIF('Raw Scores'!J2:J76,4)</f>
         <v>0</v>
       </c>
       <c r="E28" s="15" t="n">
-        <f aca="false">COUNTIF('Raw Scores'!H2:H76,4)</f>
+        <f aca="false">COUNTIF('Raw Scores'!K2:K76,4)</f>
         <v>0</v>
       </c>
     </row>
@@ -3488,167 +3796,274 @@
         <v>5</v>
       </c>
       <c r="B29" s="15" t="n">
-        <f aca="false">COUNTIF('Raw Scores'!E2:E76,5)</f>
-        <v>0</v>
-      </c>
-      <c r="C29" s="15" t="n">
-        <f aca="false">COUNTIF('Raw Scores'!F2:F76,5)</f>
-        <v>0</v>
-      </c>
-      <c r="D29" s="15" t="n">
-        <f aca="false">COUNTIF('Raw Scores'!G2:G76,5)</f>
-        <v>0</v>
-      </c>
-      <c r="E29" s="15" t="n">
         <f aca="false">COUNTIF('Raw Scores'!H2:H76,5)</f>
         <v>0</v>
       </c>
+      <c r="C29" s="15" t="n">
+        <f aca="false">COUNTIF('Raw Scores'!I2:I76,5)</f>
+        <v>0</v>
+      </c>
+      <c r="D29" s="15" t="n">
+        <f aca="false">COUNTIF('Raw Scores'!J2:J76,5)</f>
+        <v>0</v>
+      </c>
+      <c r="E29" s="15" t="n">
+        <f aca="false">COUNTIF('Raw Scores'!K2:K76,5)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B33" s="15" t="str">
-        <f aca="false">IFERROR(AVERAGEIFS('Raw Scores'!K$2:K$76,'Raw Scores'!B$2:B$76,A33),"")</f>
+        <f aca="false">IFERROR(AVERAGEIFS('Raw Scores'!N$2:N$76,'Raw Scores'!B$2:B$76,A33),"")</f>
         <v/>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="6" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B34" s="15" t="str">
-        <f aca="false">IFERROR(AVERAGEIFS('Raw Scores'!K$2:K$76,'Raw Scores'!B$2:B$76,A34),"")</f>
+        <f aca="false">IFERROR(AVERAGEIFS('Raw Scores'!N$2:N$76,'Raw Scores'!B$2:B$76,A34),"")</f>
         <v/>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="6" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B35" s="15" t="str">
-        <f aca="false">IFERROR(AVERAGEIFS('Raw Scores'!K$2:K$76,'Raw Scores'!B$2:B$76,A35),"")</f>
+        <f aca="false">IFERROR(AVERAGEIFS('Raw Scores'!N$2:N$76,'Raw Scores'!B$2:B$76,A35),"")</f>
         <v/>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="6" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B36" s="15" t="str">
-        <f aca="false">IFERROR(AVERAGEIFS('Raw Scores'!K$2:K$76,'Raw Scores'!B$2:B$76,A36),"")</f>
+        <f aca="false">IFERROR(AVERAGEIFS('Raw Scores'!N$2:N$76,'Raw Scores'!B$2:B$76,A36),"")</f>
         <v/>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="6" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B37" s="15" t="str">
-        <f aca="false">IFERROR(AVERAGEIFS('Raw Scores'!K$2:K$76,'Raw Scores'!B$2:B$76,A37),"")</f>
+        <f aca="false">IFERROR(AVERAGEIFS('Raw Scores'!N$2:N$76,'Raw Scores'!B$2:B$76,A37),"")</f>
         <v/>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="6" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B38" s="15" t="str">
-        <f aca="false">IFERROR(AVERAGEIFS('Raw Scores'!K$2:K$76,'Raw Scores'!B$2:B$76,A38),"")</f>
+        <f aca="false">IFERROR(AVERAGEIFS('Raw Scores'!N$2:N$76,'Raw Scores'!B$2:B$76,A38),"")</f>
         <v/>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="6" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B39" s="15" t="str">
-        <f aca="false">IFERROR(AVERAGEIFS('Raw Scores'!K$2:K$76,'Raw Scores'!B$2:B$76,A39),"")</f>
+        <f aca="false">IFERROR(AVERAGEIFS('Raw Scores'!N$2:N$76,'Raw Scores'!B$2:B$76,A39),"")</f>
         <v/>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="6" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B40" s="15" t="str">
-        <f aca="false">IFERROR(AVERAGEIFS('Raw Scores'!K$2:K$76,'Raw Scores'!B$2:B$76,A40),"")</f>
+        <f aca="false">IFERROR(AVERAGEIFS('Raw Scores'!N$2:N$76,'Raw Scores'!B$2:B$76,A40),"")</f>
         <v/>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="6" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B41" s="15" t="str">
-        <f aca="false">IFERROR(AVERAGEIFS('Raw Scores'!K$2:K$76,'Raw Scores'!B$2:B$76,A41),"")</f>
+        <f aca="false">IFERROR(AVERAGEIFS('Raw Scores'!N$2:N$76,'Raw Scores'!B$2:B$76,A41),"")</f>
         <v/>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="6" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B42" s="15" t="str">
-        <f aca="false">IFERROR(AVERAGEIFS('Raw Scores'!K$2:K$76,'Raw Scores'!B$2:B$76,A42),"")</f>
+        <f aca="false">IFERROR(AVERAGEIFS('Raw Scores'!N$2:N$76,'Raw Scores'!B$2:B$76,A42),"")</f>
         <v/>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="6" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B43" s="15" t="str">
-        <f aca="false">IFERROR(AVERAGEIFS('Raw Scores'!K$2:K$76,'Raw Scores'!B$2:B$76,A43),"")</f>
+        <f aca="false">IFERROR(AVERAGEIFS('Raw Scores'!N$2:N$76,'Raw Scores'!B$2:B$76,A43),"")</f>
         <v/>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B44" s="15" t="str">
-        <f aca="false">IFERROR(AVERAGEIFS('Raw Scores'!K$2:K$76,'Raw Scores'!B$2:B$76,A44),"")</f>
+        <f aca="false">IFERROR(AVERAGEIFS('Raw Scores'!N$2:N$76,'Raw Scores'!B$2:B$76,A44),"")</f>
         <v/>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B45" s="15" t="str">
-        <f aca="false">IFERROR(AVERAGEIFS('Raw Scores'!K$2:K$76,'Raw Scores'!B$2:B$76,A45),"")</f>
+        <f aca="false">IFERROR(AVERAGEIFS('Raw Scores'!N$2:N$76,'Raw Scores'!B$2:B$76,A45),"")</f>
         <v/>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B46" s="15" t="str">
-        <f aca="false">IFERROR(AVERAGEIFS('Raw Scores'!K$2:K$76,'Raw Scores'!B$2:B$76,A46),"")</f>
+        <f aca="false">IFERROR(AVERAGEIFS('Raw Scores'!N$2:N$76,'Raw Scores'!B$2:B$76,A46),"")</f>
         <v/>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="6" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B47" s="15" t="str">
-        <f aca="false">IFERROR(AVERAGEIFS('Raw Scores'!K$2:K$76,'Raw Scores'!B$2:B$76,A47),"")</f>
+        <f aca="false">IFERROR(AVERAGEIFS('Raw Scores'!N$2:N$76,'Raw Scores'!B$2:B$76,A47),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="4" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B50" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B51" s="15" t="n">
+        <f aca="false">COUNTIF('Raw Scores'!E$2:E$76,A51)</f>
+        <v>0</v>
+      </c>
+      <c r="C51" s="15" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Raw Scores'!N$2:N$76,'Raw Scores'!E$2:E$76,A51),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="B52" s="15" t="n">
+        <f aca="false">COUNTIF('Raw Scores'!E$2:E$76,A52)</f>
+        <v>0</v>
+      </c>
+      <c r="C52" s="15" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Raw Scores'!N$2:N$76,'Raw Scores'!E$2:E$76,A52),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="B53" s="15" t="n">
+        <f aca="false">COUNTIF('Raw Scores'!E$2:E$76,A53)</f>
+        <v>0</v>
+      </c>
+      <c r="C53" s="15" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Raw Scores'!N$2:N$76,'Raw Scores'!E$2:E$76,A53),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="B54" s="15" t="n">
+        <f aca="false">COUNTIF('Raw Scores'!E$2:E$76,A54)</f>
+        <v>0</v>
+      </c>
+      <c r="C54" s="15" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Raw Scores'!N$2:N$76,'Raw Scores'!E$2:E$76,A54),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B55" s="15" t="n">
+        <f aca="false">COUNTIF('Raw Scores'!E$2:E$76,A55)</f>
+        <v>0</v>
+      </c>
+      <c r="C55" s="15" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Raw Scores'!N$2:N$76,'Raw Scores'!E$2:E$76,A55),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="B56" s="15" t="n">
+        <f aca="false">COUNTIF('Raw Scores'!E$2:E$76,A56)</f>
+        <v>0</v>
+      </c>
+      <c r="C56" s="15" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Raw Scores'!N$2:N$76,'Raw Scores'!E$2:E$76,A56),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="B57" s="15" t="n">
+        <f aca="false">COUNTIF('Raw Scores'!E$2:E$76,A57)</f>
+        <v>0</v>
+      </c>
+      <c r="C57" s="15" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Raw Scores'!N$2:N$76,'Raw Scores'!E$2:E$76,A57),"")</f>
         <v/>
       </c>
     </row>

</xml_diff>